<commit_message>
Updated Sprint 2 Backlog & Sprint 1 Retrospective
I updated the sprint 2 backlog with the remaining tasks for the rest of
the sprint.
I added the tasks for sprint 2 to the sprint retrospective.
</commit_message>
<xml_diff>
--- a/sprints/sprint2/Sprint Backlog & Burnup Chart.xlsx
+++ b/sprints/sprint2/Sprint Backlog & Burnup Chart.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://westga365-my.sharepoint.com/personal/jcorley_westga_edu/Documents/Teaching/Software Engineering II/SE2 - Spring 2026/Project/SE2-project-repos-sample/sprints/sprint1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\College Docs\Software Engineering II\Project\Group5NutritionTracker\sprints\sprint2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{9C9C4265-351C-41A0-89E5-93A08D9C51A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C68B4513-1541-415B-8F23-00764467EF2F}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35244743-0280-48E6-AB5D-F4D32C4F2F67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="58">
   <si>
     <t>Related User Story</t>
   </si>
@@ -65,10 +65,151 @@
     <t>Estimate Totals</t>
   </si>
   <si>
-    <t>Code Things…</t>
-  </si>
-  <si>
-    <t>That User Story</t>
+    <t>Login</t>
+  </si>
+  <si>
+    <t>Login UI Page</t>
+  </si>
+  <si>
+    <t>Authorization Process Client Side</t>
+  </si>
+  <si>
+    <t>Authorization Process Server Side</t>
+  </si>
+  <si>
+    <t>Login Page Codebehind</t>
+  </si>
+  <si>
+    <t>Display logged in user's info on landing page</t>
+  </si>
+  <si>
+    <t>User Class structure</t>
+  </si>
+  <si>
+    <t>Communication Protecol for authorization process</t>
+  </si>
+  <si>
+    <t>Assigned To</t>
+  </si>
+  <si>
+    <t>Team</t>
+  </si>
+  <si>
+    <t>Create Account</t>
+  </si>
+  <si>
+    <t>Create Account UI Page</t>
+  </si>
+  <si>
+    <t>Create Account Page Code Behind</t>
+  </si>
+  <si>
+    <t>Display User Info on Landing After Creation</t>
+  </si>
+  <si>
+    <t>Communication Protecol for Create Account</t>
+  </si>
+  <si>
+    <t>Add Food Item To A Day</t>
+  </si>
+  <si>
+    <t>Fix UI Spacing Issues</t>
+  </si>
+  <si>
+    <t>Search Process Client Side</t>
+  </si>
+  <si>
+    <t>Search Process Server Side</t>
+  </si>
+  <si>
+    <t>DayOfFood Structure</t>
+  </si>
+  <si>
+    <t>Hookup Remove Buttons to User</t>
+  </si>
+  <si>
+    <t>Credentials Structure</t>
+  </si>
+  <si>
+    <t>Communication Protecol for Search</t>
+  </si>
+  <si>
+    <t>Update DayOfFood Process Client Side</t>
+  </si>
+  <si>
+    <t>Update DayOfFood Process Server Side</t>
+  </si>
+  <si>
+    <t>Communication Protecol for Update DayOfFood</t>
+  </si>
+  <si>
+    <t>Hookup Add Buttons to Search Page</t>
+  </si>
+  <si>
+    <t>Yeni</t>
+  </si>
+  <si>
+    <t>Justin</t>
+  </si>
+  <si>
+    <t>Emi</t>
+  </si>
+  <si>
+    <t>Victor</t>
+  </si>
+  <si>
+    <t>Person</t>
+  </si>
+  <si>
+    <t>Current Hours</t>
+  </si>
+  <si>
+    <t>Total Hours For Sprint</t>
+  </si>
+  <si>
+    <t>Difference</t>
+  </si>
+  <si>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>Edit Diet</t>
+  </si>
+  <si>
+    <t>Edit Diet UI Page</t>
+  </si>
+  <si>
+    <t>Edit Diet Codebehind</t>
+  </si>
+  <si>
+    <t>Edit Diet Process Client Side</t>
+  </si>
+  <si>
+    <t>Edit Diet Process Server Side</t>
+  </si>
+  <si>
+    <t>Communication Protecol for Update Diet</t>
+  </si>
+  <si>
+    <t>Create Food</t>
+  </si>
+  <si>
+    <t>Create Food Process Client Side</t>
+  </si>
+  <si>
+    <t>Create Food Process Server Side</t>
+  </si>
+  <si>
+    <t>Communication Protecol for Create Food</t>
+  </si>
+  <si>
+    <t>Create Account Process Client Side</t>
+  </si>
+  <si>
+    <t>Create Account Process Server Side</t>
+  </si>
+  <si>
+    <t>Account Menu UI</t>
   </si>
 </sst>
 </file>
@@ -92,7 +233,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -102,12 +243,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -129,8 +264,26 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.34998626667073579"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -138,23 +291,81 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -266,21 +477,21 @@
           </c:marker>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$D$27:$G$27</c:f>
+              <c:f>Sheet1!$F$37:$I$37</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>25</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>50</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>75</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>100</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -309,21 +520,21 @@
           </c:marker>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$D$28:$G$28</c:f>
+              <c:f>Sheet1!$F$38:$I$38</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>87.25</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>100</c:v>
+                  <c:v>87.25</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>100</c:v>
+                  <c:v>87.25</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>100</c:v>
+                  <c:v>87.25</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1065,15 +1276,15 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
+      <xdr:col>10</xdr:col>
       <xdr:colOff>38100</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>100012</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
+      <xdr:col>17</xdr:col>
       <xdr:colOff>342900</xdr:colOff>
-      <xdr:row>17</xdr:row>
+      <xdr:row>21</xdr:row>
       <xdr:rowOff>176212</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -1365,327 +1576,911 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:I45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="51.42578125" customWidth="1"/>
-    <col min="2" max="2" width="41.7109375" customWidth="1"/>
-    <col min="3" max="3" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.5703125" customWidth="1"/>
+    <col min="3" max="3" width="51.42578125" customWidth="1"/>
+    <col min="4" max="4" width="44" customWidth="1"/>
+    <col min="5" max="5" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="C1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="D1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="E1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="F1" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="7"/>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="5" t="s">
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="12"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="G2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="H2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="I2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="9">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="6">
+        <v>0.75</v>
+      </c>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="9">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="6">
+        <v>0.25</v>
+      </c>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" s="6">
+        <v>4</v>
+      </c>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="6">
+        <v>4</v>
+      </c>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="6">
+        <v>2.5</v>
+      </c>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="E8" s="6">
+        <v>2.75</v>
+      </c>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B9" s="9">
+        <v>1.3</v>
+      </c>
+      <c r="C9" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="1">
-        <v>100</v>
-      </c>
-      <c r="D3" s="2">
+      <c r="D9" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" s="6">
+        <v>4</v>
+      </c>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="9">
+        <v>2.1</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="E10" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="9">
+        <v>2.1</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="E11" s="6">
+        <v>0.25</v>
+      </c>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B12" s="9">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="E12" s="6">
+        <v>2.75</v>
+      </c>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B13" s="9">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="E13" s="6">
+        <v>4</v>
+      </c>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="9">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="E14" s="6">
+        <v>4</v>
+      </c>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" s="9">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="E15" s="6">
+        <v>2.5</v>
+      </c>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B16" s="9">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="E16" s="6">
+        <v>4</v>
+      </c>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" s="9">
+        <v>3.2</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="E17" s="6">
+        <v>4</v>
+      </c>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3"/>
+      <c r="I17" s="3"/>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B18" s="9">
+        <v>3.2</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="E18" s="6">
+        <v>4</v>
+      </c>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3"/>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="9">
+        <v>3.1</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="E19" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3"/>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B20" s="9">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="E20" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="3"/>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" s="9">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E21" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B22" s="9">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="E22" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="3"/>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B23" s="9">
+        <v>4.2</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D23" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E23" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="3"/>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B24" s="9">
+        <v>4.2</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E24" s="6">
+        <v>3</v>
+      </c>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B25" s="9">
+        <v>4.2</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="E25" s="6">
+        <v>3</v>
+      </c>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B26" s="9">
+        <v>4.2</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E26" s="6">
+        <v>4</v>
+      </c>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+      <c r="I26" s="3"/>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B27" s="9">
+        <v>4.2</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D27" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="E27" s="6">
+        <v>4</v>
+      </c>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="3"/>
+      <c r="I27" s="3"/>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B28" s="9">
+        <v>4.3</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="E28" s="6">
+        <v>4</v>
+      </c>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+      <c r="I28" s="3"/>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B29" s="9">
+        <v>4.3</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D29" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="E29" s="6">
+        <v>4</v>
+      </c>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="3"/>
+      <c r="I29" s="3"/>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B30" s="9">
+        <v>5.2</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D30" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="E30" s="6">
+        <v>2</v>
+      </c>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
+      <c r="H30" s="3"/>
+      <c r="I30" s="3"/>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B31" s="9">
+        <v>5.2</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D31" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="E31" s="6">
+        <v>5</v>
+      </c>
+      <c r="F31" s="3"/>
+      <c r="G31" s="3"/>
+      <c r="H31" s="3"/>
+      <c r="I31" s="3"/>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B32" s="9">
+        <v>5.3</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D32" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="E32" s="6">
+        <v>3</v>
+      </c>
+      <c r="F32" s="3"/>
+      <c r="G32" s="3"/>
+      <c r="H32" s="3"/>
+      <c r="I32" s="3"/>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B33" s="9">
+        <v>5.2</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="E33" s="6">
+        <v>4</v>
+      </c>
+      <c r="F33" s="3"/>
+      <c r="G33" s="3"/>
+      <c r="H33" s="3"/>
+      <c r="I33" s="3"/>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B34" s="9">
+        <v>5.2</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D34" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="E34" s="6">
+        <v>4</v>
+      </c>
+      <c r="F34" s="3"/>
+      <c r="G34" s="3"/>
+      <c r="H34" s="3"/>
+      <c r="I34" s="3"/>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B35" s="9">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D35" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="F3" s="2">
-        <v>75</v>
-      </c>
-      <c r="G3" s="2">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="1"/>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="1"/>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="1"/>
-      <c r="B25" s="1"/>
-      <c r="C25" s="1"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="1"/>
-      <c r="B26" s="1"/>
-      <c r="C26" s="1"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B27" s="4" t="s">
+      <c r="E35" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="F35" s="3"/>
+      <c r="G35" s="3"/>
+      <c r="H35" s="3"/>
+      <c r="I35" s="3"/>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36" s="6"/>
+      <c r="B36" s="9"/>
+      <c r="C36" s="6"/>
+      <c r="D36" s="9"/>
+      <c r="E36" s="6"/>
+      <c r="F36" s="3"/>
+      <c r="G36" s="3"/>
+      <c r="H36" s="3"/>
+      <c r="I36" s="3"/>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37" s="2"/>
+      <c r="B37" s="2"/>
+      <c r="C37" s="2"/>
+      <c r="D37" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C27" s="3">
-        <f>SUM(C3:C26)</f>
-        <v>100</v>
-      </c>
-      <c r="D27" s="3">
-        <f t="shared" ref="D27:G27" si="0">SUM(D3:D26)</f>
-        <v>25</v>
-      </c>
-      <c r="E27" s="3">
+      <c r="E37" s="5">
+        <f>SUM(E3:E36)</f>
+        <v>87.25</v>
+      </c>
+      <c r="F37" s="5">
+        <f>SUM(F3:F36)</f>
+        <v>0</v>
+      </c>
+      <c r="G37" s="5">
+        <f>SUM(G3:G36)</f>
+        <v>0</v>
+      </c>
+      <c r="H37" s="5">
+        <f>SUM(H3:H36)</f>
+        <v>0</v>
+      </c>
+      <c r="I37" s="5">
+        <f>SUM(I3:I36)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E38">
+        <v>96</v>
+      </c>
+      <c r="F38">
+        <f>$E$37</f>
+        <v>87.25</v>
+      </c>
+      <c r="G38">
+        <f t="shared" ref="G38:I38" si="0">$E$37</f>
+        <v>87.25</v>
+      </c>
+      <c r="H38">
         <f t="shared" si="0"/>
-        <v>50</v>
-      </c>
-      <c r="F27" s="3">
+        <v>87.25</v>
+      </c>
+      <c r="I38">
         <f t="shared" si="0"/>
-        <v>75</v>
-      </c>
-      <c r="G27" s="3">
-        <f t="shared" si="0"/>
-        <v>100</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="D28">
-        <f>$C$27</f>
-        <v>100</v>
-      </c>
-      <c r="E28">
-        <f t="shared" ref="E28:G28" si="1">$C$27</f>
-        <v>100</v>
-      </c>
-      <c r="F28">
-        <f t="shared" si="1"/>
-        <v>100</v>
-      </c>
-      <c r="G28">
-        <f t="shared" si="1"/>
-        <v>100</v>
+        <v>87.25</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="D40" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="E40" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="F40" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="G40" s="7" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="D41" t="s">
+        <v>37</v>
+      </c>
+      <c r="E41">
+        <f>SUMIF(A3:A36, D41,E3:E36)</f>
+        <v>19</v>
+      </c>
+      <c r="F41">
+        <v>24</v>
+      </c>
+      <c r="G41">
+        <f>F41-E41-E45</f>
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="D42" t="s">
+        <v>38</v>
+      </c>
+      <c r="E42">
+        <f>SUMIF(A3:A36, D42,E3:E36)</f>
+        <v>21.25</v>
+      </c>
+      <c r="F42">
+        <v>24</v>
+      </c>
+      <c r="G42">
+        <f>F42-E42-E45</f>
+        <v>-1.5</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="D43" t="s">
+        <v>36</v>
+      </c>
+      <c r="E43">
+        <f>SUMIF(A3:A36, D43,E3:E36)</f>
+        <v>21.75</v>
+      </c>
+      <c r="F43">
+        <v>24</v>
+      </c>
+      <c r="G43">
+        <f>F43-E43-E45</f>
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="D44" t="s">
+        <v>39</v>
+      </c>
+      <c r="E44">
+        <f>SUMIF(A3:A36, D44,E3:E36)</f>
+        <v>21</v>
+      </c>
+      <c r="F44">
+        <v>24</v>
+      </c>
+      <c r="G44">
+        <f>F44-E44-E45</f>
+        <v>-1.25</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="D45" t="s">
+        <v>18</v>
+      </c>
+      <c r="E45">
+        <f>SUMIF(A3:A36, D45,E3:E36)</f>
+        <v>4.25</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="D1:G1"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:E36">
+    <sortCondition ref="B3:B36"/>
+    <sortCondition ref="D3:D36"/>
+  </sortState>
+  <mergeCells count="6">
+    <mergeCell ref="F1:I1"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="D1:D2"/>
     <mergeCell ref="C1:C2"/>
+    <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
-    <mergeCell ref="A1:A2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Implemented Server Client and Login Auth
I updated the Python project to include model classes for food items
Added food items to the python database.
Fixed python server issues with Json string building. Used ChatGPT
to troubleshoot issues with Json strings
Updated the client in the Java project to work with any string for
all requests
Updated added handling for the login authorization process to build
Json string and build user from Json string. Used ChatGPT to figure
out how to create the Json string for the request and also to help
with how to generate a user from the response Json string.
</commit_message>
<xml_diff>
--- a/sprints/sprint2/Sprint Backlog & Burnup Chart.xlsx
+++ b/sprints/sprint2/Sprint Backlog & Burnup Chart.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\College Docs\Software Engineering II\Project\Group5NutritionTracker\sprints\sprint2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\OneDrive\Documents\College Docs\Software Engineering II\Project\Group5NutritionTracker\sprints\sprint2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35244743-0280-48E6-AB5D-F4D32C4F2F67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C816719-D512-4BE4-A2F0-38D39455C072}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="59">
   <si>
     <t>Related User Story</t>
   </si>
@@ -210,6 +210,9 @@
   </si>
   <si>
     <t>Account Menu UI</t>
+  </si>
+  <si>
+    <t>Completed By</t>
   </si>
 </sst>
 </file>
@@ -336,7 +339,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -367,6 +370,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -477,12 +486,12 @@
           </c:marker>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$F$37:$I$37</c:f>
+              <c:f>Sheet1!$G$37:$J$37</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -520,7 +529,7 @@
           </c:marker>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$F$38:$I$38</c:f>
+              <c:f>Sheet1!$G$38:$J$38</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -1276,13 +1285,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>10</xdr:col>
+      <xdr:col>11</xdr:col>
       <xdr:colOff>38100</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>100012</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>17</xdr:col>
+      <xdr:col>18</xdr:col>
       <xdr:colOff>342900</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>176212</xdr:rowOff>
@@ -1576,781 +1585,819 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I45"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:J45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.5703125" customWidth="1"/>
-    <col min="3" max="3" width="51.42578125" customWidth="1"/>
-    <col min="4" max="4" width="44" customWidth="1"/>
-    <col min="5" max="5" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.85546875" customWidth="1"/>
+    <col min="1" max="1" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.21875" customWidth="1"/>
+    <col min="3" max="3" width="11.5546875" customWidth="1"/>
+    <col min="4" max="4" width="51.44140625" customWidth="1"/>
+    <col min="5" max="5" width="44" customWidth="1"/>
+    <col min="6" max="6" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="C1" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="D1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="E1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="F1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="G1" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="10"/>
       <c r="H1" s="10"/>
       <c r="I1" s="10"/>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J1" s="10"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="12"/>
-      <c r="B2" s="14"/>
-      <c r="C2" s="11"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="14"/>
       <c r="D2" s="11"/>
       <c r="E2" s="11"/>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="11"/>
+      <c r="G2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="6"/>
+      <c r="C3" s="9">
         <v>1.1000000000000001</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="D3" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="E3" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="6">
+      <c r="F3" s="6">
         <v>0.75</v>
       </c>
-      <c r="F3" s="3"/>
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J3" s="3"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="6"/>
+      <c r="C4" s="9">
         <v>1.1000000000000001</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="D4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="E4" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="6">
+      <c r="F4" s="6">
         <v>0.25</v>
       </c>
-      <c r="F4" s="3"/>
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J4" s="3"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="9">
+      <c r="B5" s="6"/>
+      <c r="C5" s="9">
         <v>1.2</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="D5" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="E5" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="6">
+      <c r="F5" s="6">
         <v>4</v>
       </c>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
+      <c r="G5" s="3">
+        <v>4</v>
+      </c>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J5" s="3"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="6"/>
+      <c r="C6" s="9">
         <v>1.2</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="D6" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="E6" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="6">
+      <c r="F6" s="6">
         <v>4</v>
       </c>
-      <c r="F6" s="3"/>
       <c r="G6" s="3"/>
       <c r="H6" s="3"/>
       <c r="I6" s="3"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J6" s="3"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B7" s="9">
+      <c r="B7" s="6"/>
+      <c r="C7" s="9">
         <v>1.2</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="D7" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="E7" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="6">
+      <c r="F7" s="6">
         <v>2.5</v>
       </c>
-      <c r="F7" s="3"/>
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J7" s="3"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B8" s="9">
+      <c r="B8" s="6"/>
+      <c r="C8" s="9">
         <v>1.2</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="D8" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="E8" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="6">
+      <c r="F8" s="6">
         <v>2.75</v>
       </c>
-      <c r="F8" s="3"/>
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J8" s="3"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B9" s="9">
+      <c r="B9" s="6"/>
+      <c r="C9" s="9">
         <v>1.3</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="D9" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="E9" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="E9" s="6">
+      <c r="F9" s="6">
         <v>4</v>
       </c>
-      <c r="F9" s="3"/>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J9" s="3"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="9">
+      <c r="B10" s="6"/>
+      <c r="C10" s="9">
         <v>2.1</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="D10" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="E10" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E10" s="6">
+      <c r="F10" s="6">
         <v>0.5</v>
       </c>
-      <c r="F10" s="3"/>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J10" s="3"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="9">
+      <c r="B11" s="6"/>
+      <c r="C11" s="9">
         <v>2.1</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="D11" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="9" t="s">
+      <c r="E11" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="E11" s="6">
+      <c r="F11" s="6">
         <v>0.25</v>
       </c>
-      <c r="F11" s="3"/>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J11" s="3"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="9">
+      <c r="B12" s="6"/>
+      <c r="C12" s="9">
         <v>2.2000000000000002</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="D12" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D12" s="9" t="s">
+      <c r="E12" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="E12" s="6">
+      <c r="F12" s="6">
         <v>2.75</v>
       </c>
-      <c r="F12" s="3"/>
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
       <c r="I12" s="3"/>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J12" s="3"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B13" s="9">
+      <c r="B13" s="6"/>
+      <c r="C13" s="9">
         <v>2.2000000000000002</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="D13" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D13" s="9" t="s">
+      <c r="E13" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="E13" s="6">
+      <c r="F13" s="6">
         <v>4</v>
       </c>
-      <c r="F13" s="3"/>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J13" s="3"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B14" s="9">
+      <c r="B14" s="6"/>
+      <c r="C14" s="9">
         <v>2.2000000000000002</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="D14" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="E14" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="E14" s="6">
+      <c r="F14" s="6">
         <v>4</v>
       </c>
-      <c r="F14" s="3"/>
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
       <c r="I14" s="3"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J14" s="3"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B15" s="9">
+      <c r="B15" s="6"/>
+      <c r="C15" s="9">
         <v>2.2000000000000002</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="D15" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D15" s="9" t="s">
+      <c r="E15" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="E15" s="6">
+      <c r="F15" s="6">
         <v>2.5</v>
       </c>
-      <c r="F15" s="3"/>
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
       <c r="I15" s="3"/>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J15" s="3"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B16" s="9">
+      <c r="B16" s="6"/>
+      <c r="C16" s="9">
         <v>2.2999999999999998</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="D16" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D16" s="9" t="s">
+      <c r="E16" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="E16" s="6">
+      <c r="F16" s="6">
         <v>4</v>
       </c>
-      <c r="F16" s="3"/>
       <c r="G16" s="3"/>
       <c r="H16" s="3"/>
       <c r="I16" s="3"/>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J16" s="3"/>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B17" s="9">
+      <c r="B17" s="6"/>
+      <c r="C17" s="9">
         <v>3.2</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="D17" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="D17" s="9" t="s">
+      <c r="E17" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="E17" s="6">
+      <c r="F17" s="6">
         <v>4</v>
       </c>
-      <c r="F17" s="3"/>
       <c r="G17" s="3"/>
       <c r="H17" s="3"/>
       <c r="I17" s="3"/>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J17" s="3"/>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B18" s="9">
+      <c r="B18" s="6"/>
+      <c r="C18" s="9">
         <v>3.2</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="D18" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="D18" s="9" t="s">
+      <c r="E18" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="E18" s="6">
+      <c r="F18" s="6">
         <v>4</v>
       </c>
-      <c r="F18" s="3"/>
       <c r="G18" s="3"/>
       <c r="H18" s="3"/>
       <c r="I18" s="3"/>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J18" s="3"/>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="9">
+      <c r="B19" s="6"/>
+      <c r="C19" s="9">
         <v>3.1</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="D19" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="D19" s="9" t="s">
+      <c r="E19" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="E19" s="6">
+      <c r="F19" s="6">
         <v>0.5</v>
       </c>
-      <c r="F19" s="3"/>
       <c r="G19" s="3"/>
       <c r="H19" s="3"/>
       <c r="I19" s="3"/>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J19" s="3"/>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="9">
+      <c r="B20" s="6"/>
+      <c r="C20" s="9">
         <v>4.0999999999999996</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="D20" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="D20" s="9" t="s">
+      <c r="E20" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="E20" s="6">
+      <c r="F20" s="6">
         <v>0.5</v>
       </c>
-      <c r="F20" s="3"/>
       <c r="G20" s="3"/>
       <c r="H20" s="3"/>
       <c r="I20" s="3"/>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J20" s="3"/>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B21" s="9">
+      <c r="B21" s="6"/>
+      <c r="C21" s="9">
         <v>4.0999999999999996</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="D21" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="D21" s="9" t="s">
+      <c r="E21" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="E21" s="6">
+      <c r="F21" s="6">
         <v>0.5</v>
       </c>
-      <c r="F21" s="3"/>
       <c r="G21" s="3"/>
       <c r="H21" s="3"/>
       <c r="I21" s="3"/>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J21" s="3"/>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B22" s="9">
+      <c r="B22" s="6"/>
+      <c r="C22" s="9">
         <v>4.0999999999999996</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="D22" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="D22" s="9" t="s">
+      <c r="E22" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="E22" s="6">
+      <c r="F22" s="6">
         <v>0.5</v>
       </c>
-      <c r="F22" s="3"/>
       <c r="G22" s="3"/>
       <c r="H22" s="3"/>
       <c r="I22" s="3"/>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J22" s="3"/>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B23" s="9">
+      <c r="B23" s="6"/>
+      <c r="C23" s="9">
         <v>4.2</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="D23" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="D23" s="9" t="s">
+      <c r="E23" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="E23" s="6">
+      <c r="F23" s="6">
         <v>0.5</v>
       </c>
-      <c r="F23" s="3"/>
       <c r="G23" s="3"/>
       <c r="H23" s="3"/>
       <c r="I23" s="3"/>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J23" s="3"/>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B24" s="9">
+      <c r="B24" s="6"/>
+      <c r="C24" s="9">
         <v>4.2</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="D24" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="D24" s="9" t="s">
+      <c r="E24" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="E24" s="6">
+      <c r="F24" s="6">
         <v>3</v>
       </c>
-      <c r="F24" s="3"/>
       <c r="G24" s="3"/>
       <c r="H24" s="3"/>
       <c r="I24" s="3"/>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J24" s="3"/>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B25" s="9">
+      <c r="B25" s="6"/>
+      <c r="C25" s="9">
         <v>4.2</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="D25" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="D25" s="9" t="s">
+      <c r="E25" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="E25" s="6">
+      <c r="F25" s="6">
         <v>3</v>
       </c>
-      <c r="F25" s="3"/>
       <c r="G25" s="3"/>
       <c r="H25" s="3"/>
       <c r="I25" s="3"/>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J25" s="3"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B26" s="9">
+      <c r="B26" s="6"/>
+      <c r="C26" s="9">
         <v>4.2</v>
       </c>
-      <c r="C26" s="6" t="s">
+      <c r="D26" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="D26" s="9" t="s">
+      <c r="E26" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="E26" s="6">
+      <c r="F26" s="6">
         <v>4</v>
       </c>
-      <c r="F26" s="3"/>
       <c r="G26" s="3"/>
       <c r="H26" s="3"/>
       <c r="I26" s="3"/>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J26" s="3"/>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B27" s="9">
+      <c r="B27" s="6"/>
+      <c r="C27" s="9">
         <v>4.2</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="D27" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="D27" s="9" t="s">
+      <c r="E27" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="E27" s="6">
+      <c r="F27" s="6">
         <v>4</v>
       </c>
-      <c r="F27" s="3"/>
       <c r="G27" s="3"/>
       <c r="H27" s="3"/>
       <c r="I27" s="3"/>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J27" s="3"/>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B28" s="9">
+      <c r="B28" s="6"/>
+      <c r="C28" s="9">
         <v>4.3</v>
       </c>
-      <c r="C28" s="6" t="s">
+      <c r="D28" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="D28" s="9" t="s">
+      <c r="E28" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="E28" s="6">
+      <c r="F28" s="6">
         <v>4</v>
       </c>
-      <c r="F28" s="3"/>
       <c r="G28" s="3"/>
       <c r="H28" s="3"/>
       <c r="I28" s="3"/>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J28" s="3"/>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B29" s="9">
+      <c r="B29" s="6"/>
+      <c r="C29" s="9">
         <v>4.3</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="D29" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="D29" s="9" t="s">
+      <c r="E29" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="E29" s="6">
+      <c r="F29" s="6">
         <v>4</v>
       </c>
-      <c r="F29" s="3"/>
       <c r="G29" s="3"/>
       <c r="H29" s="3"/>
       <c r="I29" s="3"/>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J29" s="3"/>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B30" s="9">
+      <c r="B30" s="6"/>
+      <c r="C30" s="9">
         <v>5.2</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="D30" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="D30" s="9" t="s">
+      <c r="E30" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="E30" s="6">
+      <c r="F30" s="6">
         <v>2</v>
       </c>
-      <c r="F30" s="3"/>
       <c r="G30" s="3"/>
       <c r="H30" s="3"/>
       <c r="I30" s="3"/>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J30" s="3"/>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B31" s="9">
+      <c r="B31" s="6"/>
+      <c r="C31" s="9">
         <v>5.2</v>
       </c>
-      <c r="C31" s="6" t="s">
+      <c r="D31" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="D31" s="9" t="s">
+      <c r="E31" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="E31" s="6">
+      <c r="F31" s="6">
         <v>5</v>
       </c>
-      <c r="F31" s="3"/>
       <c r="G31" s="3"/>
       <c r="H31" s="3"/>
       <c r="I31" s="3"/>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J31" s="3"/>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B32" s="9">
+      <c r="B32" s="6"/>
+      <c r="C32" s="9">
         <v>5.3</v>
       </c>
-      <c r="C32" s="6" t="s">
+      <c r="D32" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="D32" s="9" t="s">
+      <c r="E32" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E32" s="6">
+      <c r="F32" s="6">
         <v>3</v>
       </c>
-      <c r="F32" s="3"/>
       <c r="G32" s="3"/>
       <c r="H32" s="3"/>
       <c r="I32" s="3"/>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J32" s="3"/>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B33" s="9">
+      <c r="B33" s="6"/>
+      <c r="C33" s="9">
         <v>5.2</v>
       </c>
-      <c r="C33" s="6" t="s">
+      <c r="D33" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="D33" s="9" t="s">
+      <c r="E33" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="E33" s="6">
+      <c r="F33" s="6">
         <v>4</v>
       </c>
-      <c r="F33" s="3"/>
       <c r="G33" s="3"/>
       <c r="H33" s="3"/>
       <c r="I33" s="3"/>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J33" s="3"/>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B34" s="9">
+      <c r="B34" s="6"/>
+      <c r="C34" s="9">
         <v>5.2</v>
       </c>
-      <c r="C34" s="6" t="s">
+      <c r="D34" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="D34" s="9" t="s">
+      <c r="E34" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="E34" s="6">
+      <c r="F34" s="6">
         <v>4</v>
       </c>
-      <c r="F34" s="3"/>
       <c r="G34" s="3"/>
       <c r="H34" s="3"/>
       <c r="I34" s="3"/>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J34" s="3"/>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B35" s="9">
+      <c r="B35" s="6"/>
+      <c r="C35" s="9">
         <v>5.0999999999999996</v>
       </c>
-      <c r="C35" s="6" t="s">
+      <c r="D35" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="D35" s="9" t="s">
+      <c r="E35" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="E35" s="6">
+      <c r="F35" s="6">
         <v>0.5</v>
       </c>
-      <c r="F35" s="3"/>
       <c r="G35" s="3"/>
       <c r="H35" s="3"/>
       <c r="I35" s="3"/>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J35" s="3"/>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" s="6"/>
-      <c r="B36" s="9"/>
-      <c r="C36" s="6"/>
-      <c r="D36" s="9"/>
-      <c r="E36" s="6"/>
-      <c r="F36" s="3"/>
+      <c r="B36" s="6"/>
+      <c r="C36" s="9"/>
+      <c r="D36" s="6"/>
+      <c r="E36" s="9"/>
+      <c r="F36" s="6"/>
       <c r="G36" s="3"/>
       <c r="H36" s="3"/>
       <c r="I36" s="3"/>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J36" s="3"/>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
-      <c r="D37" s="4" t="s">
+      <c r="D37" s="2"/>
+      <c r="E37" s="4" t="s">
         <v>8</v>
-      </c>
-      <c r="E37" s="5">
-        <f>SUM(E3:E36)</f>
-        <v>87.25</v>
       </c>
       <c r="F37" s="5">
         <f>SUM(F3:F36)</f>
-        <v>0</v>
+        <v>87.25</v>
       </c>
       <c r="G37" s="5">
         <f>SUM(G3:G36)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H37" s="5">
         <f>SUM(H3:H36)</f>
@@ -2360,126 +2407,131 @@
         <f>SUM(I3:I36)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E38">
+      <c r="J37" s="5">
+        <f>SUM(J3:J36)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="F38">
         <v>96</v>
       </c>
-      <c r="F38">
-        <f>$E$37</f>
+      <c r="G38">
+        <f>$F$37</f>
         <v>87.25</v>
       </c>
-      <c r="G38">
-        <f t="shared" ref="G38:I38" si="0">$E$37</f>
-        <v>87.25</v>
-      </c>
       <c r="H38">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="H38:J38" si="0">$F$37</f>
         <v>87.25</v>
       </c>
       <c r="I38">
         <f t="shared" si="0"/>
         <v>87.25</v>
       </c>
-    </row>
-    <row r="40" spans="1:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="D40" s="7" t="s">
+      <c r="J38">
+        <f t="shared" si="0"/>
+        <v>87.25</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="E40" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="E40" s="7" t="s">
+      <c r="F40" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="F40" s="8" t="s">
+      <c r="G40" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="G40" s="7" t="s">
+      <c r="H40" s="7" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="D41" t="s">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E41" t="s">
         <v>37</v>
       </c>
-      <c r="E41">
-        <f>SUMIF(A3:A36, D41,E3:E36)</f>
+      <c r="F41">
+        <f>SUMIF(A3:A36, E41,F3:F36)</f>
         <v>19</v>
       </c>
-      <c r="F41">
+      <c r="G41">
         <v>24</v>
       </c>
-      <c r="G41">
-        <f>F41-E41-E45</f>
+      <c r="H41">
+        <f>G41-F41-F45</f>
         <v>0.75</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="D42" t="s">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E42" t="s">
         <v>38</v>
       </c>
-      <c r="E42">
-        <f>SUMIF(A3:A36, D42,E3:E36)</f>
+      <c r="F42">
+        <f>SUMIF(A3:A36, E42,F3:F36)</f>
         <v>21.25</v>
       </c>
-      <c r="F42">
+      <c r="G42">
         <v>24</v>
       </c>
-      <c r="G42">
-        <f>F42-E42-E45</f>
+      <c r="H42">
+        <f>G42-F42-F45</f>
         <v>-1.5</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="D43" t="s">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E43" t="s">
         <v>36</v>
       </c>
-      <c r="E43">
-        <f>SUMIF(A3:A36, D43,E3:E36)</f>
+      <c r="F43">
+        <f>SUMIF(A3:A36, E43,F3:F36)</f>
         <v>21.75</v>
       </c>
-      <c r="F43">
+      <c r="G43">
         <v>24</v>
       </c>
-      <c r="G43">
-        <f>F43-E43-E45</f>
+      <c r="H43">
+        <f>G43-F43-F45</f>
         <v>-2</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="D44" t="s">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E44" t="s">
         <v>39</v>
       </c>
-      <c r="E44">
-        <f>SUMIF(A3:A36, D44,E3:E36)</f>
+      <c r="F44">
+        <f>SUMIF(A3:A36, E44,F3:F36)</f>
         <v>21</v>
       </c>
-      <c r="F44">
+      <c r="G44">
         <v>24</v>
       </c>
-      <c r="G44">
-        <f>F44-E44-E45</f>
+      <c r="H44">
+        <f>G44-F44-F45</f>
         <v>-1.25</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="D45" t="s">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E45" t="s">
         <v>18</v>
       </c>
-      <c r="E45">
-        <f>SUMIF(A3:A36, D45,E3:E36)</f>
+      <c r="F45">
+        <f>SUMIF(A3:A36, E45,F3:F36)</f>
         <v>4.25</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:E36">
-    <sortCondition ref="B3:B36"/>
-    <sortCondition ref="D3:D36"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:F36">
+    <sortCondition ref="C3:C36"/>
+    <sortCondition ref="E3:E36"/>
   </sortState>
-  <mergeCells count="6">
-    <mergeCell ref="F1:I1"/>
+  <mergeCells count="7">
+    <mergeCell ref="G1:J1"/>
+    <mergeCell ref="F1:F2"/>
     <mergeCell ref="E1:E2"/>
     <mergeCell ref="D1:D2"/>
+    <mergeCell ref="A1:A2"/>
     <mergeCell ref="C1:C2"/>
-    <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updated Sprint Backlog & Communication Protecols
Updated the sprint back log with times.
Added Communication Protecols for create account and search
</commit_message>
<xml_diff>
--- a/sprints/sprint2/Sprint Backlog & Burnup Chart.xlsx
+++ b/sprints/sprint2/Sprint Backlog & Burnup Chart.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\OneDrive\Documents\College Docs\Software Engineering II\Project\Group5NutritionTracker\sprints\sprint2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\College Docs\Software Engineering II\Project\Group5NutritionTracker\sprints\sprint2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C816719-D512-4BE4-A2F0-38D39455C072}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1753E291-32AF-401D-8137-1C4BBF78B56A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="58">
   <si>
     <t>Related User Story</t>
   </si>
@@ -104,9 +104,6 @@
     <t>Create Account Page Code Behind</t>
   </si>
   <si>
-    <t>Display User Info on Landing After Creation</t>
-  </si>
-  <si>
     <t>Communication Protecol for Create Account</t>
   </si>
   <si>
@@ -122,15 +119,9 @@
     <t>Search Process Server Side</t>
   </si>
   <si>
-    <t>DayOfFood Structure</t>
-  </si>
-  <si>
     <t>Hookup Remove Buttons to User</t>
   </si>
   <si>
-    <t>Credentials Structure</t>
-  </si>
-  <si>
     <t>Communication Protecol for Search</t>
   </si>
   <si>
@@ -140,9 +131,6 @@
     <t>Update DayOfFood Process Server Side</t>
   </si>
   <si>
-    <t>Communication Protecol for Update DayOfFood</t>
-  </si>
-  <si>
     <t>Hookup Add Buttons to Search Page</t>
   </si>
   <si>
@@ -213,6 +201,15 @@
   </si>
   <si>
     <t>Completed By</t>
+  </si>
+  <si>
+    <t>Updated To</t>
+  </si>
+  <si>
+    <t>Communication Protecol for Update FoodLog</t>
+  </si>
+  <si>
+    <t>FoodLog Structure</t>
   </si>
 </sst>
 </file>
@@ -281,7 +278,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -339,7 +336,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -355,28 +352,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -472,6 +463,9 @@
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
+          <c:tx>
+            <c:v>Actual Values</c:v>
+          </c:tx>
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
@@ -486,21 +480,21 @@
           </c:marker>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$G$37:$J$37</c:f>
+              <c:f>Sheet1!$H$35:$K$35</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>4</c:v>
+                  <c:v>4.5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>14.25</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>17.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>17.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -515,6 +509,9 @@
         <c:ser>
           <c:idx val="1"/>
           <c:order val="1"/>
+          <c:tx>
+            <c:v>Goal Line</c:v>
+          </c:tx>
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
@@ -529,21 +526,21 @@
           </c:marker>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$G$38:$J$38</c:f>
+              <c:f>Sheet1!$H$36:$K$36</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>87.25</c:v>
+                  <c:v>84.5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>87.25</c:v>
+                  <c:v>84.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>87.25</c:v>
+                  <c:v>84.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>87.25</c:v>
+                  <c:v>84.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1585,939 +1582,980 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J45"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:K43"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.21875" customWidth="1"/>
-    <col min="3" max="3" width="11.5546875" customWidth="1"/>
-    <col min="4" max="4" width="51.44140625" customWidth="1"/>
+    <col min="1" max="1" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11" customWidth="1"/>
     <col min="5" max="5" width="44" customWidth="1"/>
-    <col min="6" max="6" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.88671875" customWidth="1"/>
+    <col min="6" max="6" width="46.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="C1" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="D1" s="11" t="s">
+      <c r="B1" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="F1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="G1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="10" t="s">
+      <c r="H1" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
-      <c r="J1" s="10"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="12"/>
-      <c r="B2" s="16"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="1" t="s">
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" s="11"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="9">
+      <c r="B3" s="14"/>
+      <c r="C3" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="14">
         <v>1.1000000000000001</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="E3" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="F3" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="F3" s="6">
+      <c r="G3" s="6">
         <v>0.75</v>
       </c>
-      <c r="G3" s="3"/>
       <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
+      <c r="I3" s="3">
+        <v>0.5</v>
+      </c>
       <c r="J3" s="3"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K3" s="3"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="6"/>
-      <c r="C4" s="9">
+      <c r="B4" s="14"/>
+      <c r="C4" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="14">
         <v>1.1000000000000001</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="E4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="F4" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="F4" s="6">
+      <c r="G4" s="6">
         <v>0.25</v>
       </c>
-      <c r="G4" s="3"/>
       <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
+      <c r="I4" s="3">
+        <v>0.25</v>
+      </c>
       <c r="J4" s="3"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K4" s="3"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B5" s="6"/>
-      <c r="C5" s="9">
+        <v>34</v>
+      </c>
+      <c r="B5" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5" s="14">
         <v>1.2</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="E5" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="F5" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="6">
+      <c r="G5" s="6">
         <v>4</v>
       </c>
-      <c r="G5" s="3">
+      <c r="H5" s="3"/>
+      <c r="I5" s="3">
+        <v>6</v>
+      </c>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" s="14"/>
+      <c r="C6" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" s="14">
+        <v>1.2</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F6" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" s="6">
         <v>4</v>
       </c>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="B6" s="6"/>
-      <c r="C6" s="9">
+      <c r="H6" s="3">
+        <v>4</v>
+      </c>
+      <c r="I6" s="3">
+        <v>3</v>
+      </c>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" s="14"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="14">
         <v>1.2</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="E7" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="6">
-        <v>4</v>
-      </c>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
-      <c r="J6" s="3"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B7" s="6"/>
-      <c r="C7" s="9">
-        <v>1.2</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="E7" s="9" t="s">
+      <c r="F7" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="6">
+      <c r="G7" s="6">
         <v>2.5</v>
       </c>
-      <c r="G7" s="3"/>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K7" s="3"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="B8" s="6"/>
-      <c r="C8" s="9">
+        <v>32</v>
+      </c>
+      <c r="B8" s="14"/>
+      <c r="C8" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" s="14">
         <v>1.2</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="E8" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="F8" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="F8" s="6">
+      <c r="G8" s="6">
         <v>2.75</v>
       </c>
-      <c r="G8" s="3"/>
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
       <c r="J8" s="3"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K8" s="3"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="B9" s="6"/>
-      <c r="C9" s="9">
+        <v>32</v>
+      </c>
+      <c r="B9" s="14"/>
+      <c r="C9" s="6"/>
+      <c r="D9" s="14">
         <v>1.3</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="E9" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="F9" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="F9" s="6">
+      <c r="G9" s="6">
         <v>4</v>
       </c>
-      <c r="G9" s="3"/>
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K9" s="3"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="6"/>
-      <c r="C10" s="9">
+      <c r="B10" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" s="14">
         <v>2.1</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="E10" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E10" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="F10" s="6">
+      <c r="F10" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="G10" s="6">
         <v>0.5</v>
       </c>
-      <c r="G10" s="3"/>
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J10" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="K10" s="3"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" s="6"/>
-      <c r="C11" s="9">
-        <v>2.1</v>
-      </c>
-      <c r="D11" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" s="6"/>
+      <c r="D11" s="14">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="E11" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E11" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="F11" s="6">
-        <v>0.25</v>
-      </c>
-      <c r="G11" s="3"/>
+      <c r="F11" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="G11" s="6">
+        <v>4</v>
+      </c>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
       <c r="J11" s="3"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K11" s="3"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B12" s="6"/>
-      <c r="C12" s="9">
+        <v>32</v>
+      </c>
+      <c r="B12" s="14"/>
+      <c r="C12" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D12" s="14">
         <v>2.2000000000000002</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="E12" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E12" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="F12" s="6">
-        <v>2.75</v>
-      </c>
-      <c r="G12" s="3"/>
+      <c r="F12" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="G12" s="6">
+        <v>4</v>
+      </c>
       <c r="H12" s="3"/>
       <c r="I12" s="3"/>
       <c r="J12" s="3"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K12" s="3"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="B13" s="6"/>
-      <c r="C13" s="9">
+        <v>34</v>
+      </c>
+      <c r="B13" s="14"/>
+      <c r="C13" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D13" s="14">
         <v>2.2000000000000002</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="E13" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E13" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="F13" s="6">
-        <v>4</v>
-      </c>
-      <c r="G13" s="3"/>
+      <c r="F13" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="G13" s="6">
+        <v>2.75</v>
+      </c>
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
       <c r="J13" s="3"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K13" s="3"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="B14" s="6"/>
-      <c r="C14" s="9">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="D14" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B14" s="14"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="14">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="E14" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E14" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="F14" s="6">
+      <c r="F14" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="G14" s="6">
         <v>4</v>
       </c>
-      <c r="G14" s="3"/>
       <c r="H14" s="3"/>
       <c r="I14" s="3"/>
       <c r="J14" s="3"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K14" s="3"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B15" s="6"/>
-      <c r="C15" s="9">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E15" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="F15" s="6">
-        <v>2.5</v>
-      </c>
-      <c r="G15" s="3"/>
+        <v>18</v>
+      </c>
+      <c r="B15" s="14"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="14">
+        <v>3.1</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="F15" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="G15" s="6">
+        <v>0.5</v>
+      </c>
       <c r="H15" s="3"/>
       <c r="I15" s="3"/>
       <c r="J15" s="3"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K15" s="3"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B16" s="6"/>
-      <c r="C16" s="9">
-        <v>2.2999999999999998</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E16" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="F16" s="6">
+        <v>32</v>
+      </c>
+      <c r="B16" s="14"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="14">
+        <v>3.2</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="F16" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="G16" s="6">
         <v>4</v>
       </c>
-      <c r="G16" s="3"/>
       <c r="H16" s="3"/>
       <c r="I16" s="3"/>
       <c r="J16" s="3"/>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K16" s="3"/>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="B17" s="6"/>
-      <c r="C17" s="9">
+        <v>35</v>
+      </c>
+      <c r="B17" s="14"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="14">
         <v>3.2</v>
       </c>
-      <c r="D17" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="E17" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="F17" s="6">
+      <c r="E17" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="F17" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="G17" s="6">
         <v>4</v>
       </c>
-      <c r="G17" s="3"/>
       <c r="H17" s="3"/>
       <c r="I17" s="3"/>
       <c r="J17" s="3"/>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K17" s="3"/>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B18" s="6"/>
-      <c r="C18" s="9">
-        <v>3.2</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="E18" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="F18" s="6">
-        <v>4</v>
-      </c>
-      <c r="G18" s="3"/>
+        <v>18</v>
+      </c>
+      <c r="B18" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D18" s="14">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F18" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="G18" s="6">
+        <v>0.5</v>
+      </c>
       <c r="H18" s="3"/>
       <c r="I18" s="3"/>
-      <c r="J18" s="3"/>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J18" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="K18" s="3"/>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="6"/>
-      <c r="C19" s="9">
-        <v>3.1</v>
-      </c>
-      <c r="D19" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="E19" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="F19" s="6">
+      <c r="B19" s="14"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="14">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F19" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="G19" s="6">
         <v>0.5</v>
       </c>
-      <c r="G19" s="3"/>
       <c r="H19" s="3"/>
       <c r="I19" s="3"/>
       <c r="J19" s="3"/>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K19" s="3"/>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="6"/>
-      <c r="C20" s="9">
+      <c r="B20" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D20" s="14">
         <v>4.0999999999999996</v>
       </c>
-      <c r="D20" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E20" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="F20" s="6">
+      <c r="E20" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F20" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="G20" s="6">
         <v>0.5</v>
       </c>
-      <c r="G20" s="3"/>
-      <c r="H20" s="3"/>
+      <c r="H20" s="3">
+        <v>0.5</v>
+      </c>
       <c r="I20" s="3"/>
       <c r="J20" s="3"/>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K20" s="3"/>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B21" s="6"/>
-      <c r="C21" s="9">
-        <v>4.0999999999999996</v>
-      </c>
-      <c r="D21" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B21" s="14"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="14">
+        <v>4.2</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F21" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="E21" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="F21" s="6">
+      <c r="G21" s="6">
         <v>0.5</v>
       </c>
-      <c r="G21" s="3"/>
       <c r="H21" s="3"/>
       <c r="I21" s="3"/>
       <c r="J21" s="3"/>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K21" s="3"/>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B22" s="6"/>
-      <c r="C22" s="9">
-        <v>4.0999999999999996</v>
-      </c>
-      <c r="D22" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E22" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="F22" s="6">
-        <v>0.5</v>
-      </c>
-      <c r="G22" s="3"/>
+        <v>34</v>
+      </c>
+      <c r="B22" s="14"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="14">
+        <v>4.2</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F22" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="G22" s="6">
+        <v>3</v>
+      </c>
       <c r="H22" s="3"/>
       <c r="I22" s="3"/>
       <c r="J22" s="3"/>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K22" s="3"/>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B23" s="6"/>
-      <c r="C23" s="9">
+        <v>32</v>
+      </c>
+      <c r="B23" s="14"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="14">
         <v>4.2</v>
       </c>
-      <c r="D23" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E23" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="F23" s="6">
-        <v>0.5</v>
-      </c>
-      <c r="G23" s="3"/>
+      <c r="E23" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F23" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="G23" s="6">
+        <v>3</v>
+      </c>
       <c r="H23" s="3"/>
       <c r="I23" s="3"/>
       <c r="J23" s="3"/>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K23" s="3"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B24" s="6"/>
-      <c r="C24" s="9">
+        <v>35</v>
+      </c>
+      <c r="B24" s="14"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="14">
         <v>4.2</v>
       </c>
-      <c r="D24" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E24" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="F24" s="6">
-        <v>3</v>
-      </c>
-      <c r="G24" s="3"/>
+      <c r="E24" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F24" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="G24" s="6">
+        <v>4</v>
+      </c>
       <c r="H24" s="3"/>
       <c r="I24" s="3"/>
       <c r="J24" s="3"/>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K24" s="3"/>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="B25" s="6"/>
-      <c r="C25" s="9">
+        <v>33</v>
+      </c>
+      <c r="B25" s="14"/>
+      <c r="C25" s="6"/>
+      <c r="D25" s="14">
         <v>4.2</v>
       </c>
-      <c r="D25" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E25" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="F25" s="6">
-        <v>3</v>
-      </c>
-      <c r="G25" s="3"/>
+      <c r="E25" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F25" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="G25" s="6">
+        <v>4</v>
+      </c>
       <c r="H25" s="3"/>
       <c r="I25" s="3"/>
-      <c r="J25" s="3"/>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J25" s="3">
+        <v>2.5</v>
+      </c>
+      <c r="K25" s="3"/>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B26" s="6"/>
-      <c r="C26" s="9">
-        <v>4.2</v>
-      </c>
-      <c r="D26" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E26" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="F26" s="6">
+        <v>33</v>
+      </c>
+      <c r="B26" s="14"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="14">
+        <v>4.3</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F26" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="G26" s="6">
         <v>4</v>
       </c>
-      <c r="G26" s="3"/>
       <c r="H26" s="3"/>
       <c r="I26" s="3"/>
       <c r="J26" s="3"/>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K26" s="3"/>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="B27" s="6"/>
-      <c r="C27" s="9">
-        <v>4.2</v>
-      </c>
-      <c r="D27" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E27" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="F27" s="6">
+        <v>35</v>
+      </c>
+      <c r="B27" s="14"/>
+      <c r="C27" s="6"/>
+      <c r="D27" s="14">
+        <v>4.3</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F27" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="G27" s="6">
         <v>4</v>
       </c>
-      <c r="G27" s="3"/>
       <c r="H27" s="3"/>
       <c r="I27" s="3"/>
       <c r="J27" s="3"/>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K27" s="3"/>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="B28" s="6"/>
-      <c r="C28" s="9">
-        <v>4.3</v>
-      </c>
-      <c r="D28" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E28" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="F28" s="6">
-        <v>4</v>
-      </c>
-      <c r="G28" s="3"/>
+        <v>18</v>
+      </c>
+      <c r="B28" s="14"/>
+      <c r="C28" s="6"/>
+      <c r="D28" s="14">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="F28" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="G28" s="6">
+        <v>0.5</v>
+      </c>
       <c r="H28" s="3"/>
       <c r="I28" s="3"/>
       <c r="J28" s="3"/>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K28" s="3"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B29" s="6"/>
-      <c r="C29" s="9">
-        <v>4.3</v>
-      </c>
-      <c r="D29" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E29" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="F29" s="6">
-        <v>4</v>
-      </c>
-      <c r="G29" s="3"/>
+        <v>34</v>
+      </c>
+      <c r="B29" s="14"/>
+      <c r="C29" s="6"/>
+      <c r="D29" s="14">
+        <v>5.2</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="F29" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="G29" s="6">
+        <v>5</v>
+      </c>
       <c r="H29" s="3"/>
       <c r="I29" s="3"/>
       <c r="J29" s="3"/>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K29" s="3"/>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B30" s="6"/>
-      <c r="C30" s="9">
+        <v>35</v>
+      </c>
+      <c r="B30" s="14"/>
+      <c r="C30" s="6"/>
+      <c r="D30" s="14">
         <v>5.2</v>
       </c>
-      <c r="D30" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="E30" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="F30" s="6">
-        <v>2</v>
-      </c>
-      <c r="G30" s="3"/>
+      <c r="E30" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="F30" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="G30" s="6">
+        <v>4</v>
+      </c>
       <c r="H30" s="3"/>
       <c r="I30" s="3"/>
       <c r="J30" s="3"/>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K30" s="3"/>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B31" s="6"/>
-      <c r="C31" s="9">
+        <v>32</v>
+      </c>
+      <c r="B31" s="14"/>
+      <c r="C31" s="6"/>
+      <c r="D31" s="14">
         <v>5.2</v>
       </c>
-      <c r="D31" s="6" t="s">
+      <c r="E31" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="F31" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="E31" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="F31" s="6">
-        <v>5</v>
-      </c>
-      <c r="G31" s="3"/>
+      <c r="G31" s="6">
+        <v>4</v>
+      </c>
       <c r="H31" s="3"/>
       <c r="I31" s="3"/>
       <c r="J31" s="3"/>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K31" s="3"/>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="B32" s="6"/>
-      <c r="C32" s="9">
-        <v>5.3</v>
-      </c>
-      <c r="D32" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="E32" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="F32" s="6">
-        <v>3</v>
-      </c>
-      <c r="G32" s="3"/>
+        <v>34</v>
+      </c>
+      <c r="B32" s="14"/>
+      <c r="C32" s="6"/>
+      <c r="D32" s="14">
+        <v>5.2</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="F32" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="G32" s="6">
+        <v>2</v>
+      </c>
       <c r="H32" s="3"/>
       <c r="I32" s="3"/>
       <c r="J32" s="3"/>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K32" s="3"/>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B33" s="6"/>
-      <c r="C33" s="9">
-        <v>5.2</v>
-      </c>
-      <c r="D33" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="E33" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="F33" s="6">
-        <v>4</v>
-      </c>
-      <c r="G33" s="3"/>
+        <v>33</v>
+      </c>
+      <c r="B33" s="14"/>
+      <c r="C33" s="6"/>
+      <c r="D33" s="14">
+        <v>5.3</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="F33" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="G33" s="6">
+        <v>3</v>
+      </c>
       <c r="H33" s="3"/>
       <c r="I33" s="3"/>
       <c r="J33" s="3"/>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A34" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="B34" s="6"/>
-      <c r="C34" s="9">
-        <v>5.2</v>
-      </c>
-      <c r="D34" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="E34" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="F34" s="6">
-        <v>4</v>
-      </c>
-      <c r="G34" s="3"/>
+      <c r="K33" s="3"/>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" s="6"/>
+      <c r="B34" s="14"/>
+      <c r="C34" s="6"/>
+      <c r="D34" s="14"/>
+      <c r="E34" s="6"/>
+      <c r="F34" s="14"/>
+      <c r="G34" s="6"/>
       <c r="H34" s="3"/>
       <c r="I34" s="3"/>
       <c r="J34" s="3"/>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A35" s="6" t="s">
+      <c r="K34" s="3"/>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35" s="2"/>
+      <c r="B35" s="2"/>
+      <c r="C35" s="2"/>
+      <c r="D35" s="2"/>
+      <c r="E35" s="2"/>
+      <c r="F35" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="G35" s="5">
+        <f>SUM(G3:G34)</f>
+        <v>84.5</v>
+      </c>
+      <c r="H35" s="5">
+        <f>SUM(H3:H34)</f>
+        <v>4.5</v>
+      </c>
+      <c r="I35" s="5">
+        <f>SUM(I3:I34, H35)</f>
+        <v>14.25</v>
+      </c>
+      <c r="J35" s="5">
+        <f>SUM(J3:J34, I35)</f>
+        <v>17.5</v>
+      </c>
+      <c r="K35" s="5">
+        <f>SUM(K3:K34, J35)</f>
+        <v>17.5</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="G36">
+        <v>96</v>
+      </c>
+      <c r="H36">
+        <f>$G$35</f>
+        <v>84.5</v>
+      </c>
+      <c r="I36">
+        <f t="shared" ref="I36:K36" si="0">$G$35</f>
+        <v>84.5</v>
+      </c>
+      <c r="J36">
+        <f t="shared" si="0"/>
+        <v>84.5</v>
+      </c>
+      <c r="K36">
+        <f t="shared" si="0"/>
+        <v>84.5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="F38" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G38" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="H38" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="I38" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="J38" s="8"/>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="F39" t="s">
+        <v>33</v>
+      </c>
+      <c r="G39">
+        <f>SUMIF(A3:A34, F39,G3:G34)</f>
+        <v>19</v>
+      </c>
+      <c r="H39">
+        <v>24</v>
+      </c>
+      <c r="I39">
+        <f>H39-G39-G43</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="F40" t="s">
+        <v>34</v>
+      </c>
+      <c r="G40">
+        <f>SUMIF(A3:A34, F40,G3:G34)</f>
+        <v>21.25</v>
+      </c>
+      <c r="H40">
+        <v>24</v>
+      </c>
+      <c r="I40">
+        <f>H40-G40-G43</f>
+        <v>-1.25</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="F41" t="s">
+        <v>32</v>
+      </c>
+      <c r="G41">
+        <f>SUMIF(A3:A34, F41,G3:G34)</f>
+        <v>21.75</v>
+      </c>
+      <c r="H41">
+        <v>24</v>
+      </c>
+      <c r="I41">
+        <f>H41-G41-G43</f>
+        <v>-1.75</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="F42" t="s">
+        <v>35</v>
+      </c>
+      <c r="G42">
+        <f>SUMIF(A3:A34, F42,G3:G34)</f>
+        <v>18.5</v>
+      </c>
+      <c r="H42">
+        <v>24</v>
+      </c>
+      <c r="I42">
+        <f>H42-G42-G43</f>
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="F43" t="s">
         <v>18</v>
       </c>
-      <c r="B35" s="6"/>
-      <c r="C35" s="9">
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="D35" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="E35" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="F35" s="6">
-        <v>0.5</v>
-      </c>
-      <c r="G35" s="3"/>
-      <c r="H35" s="3"/>
-      <c r="I35" s="3"/>
-      <c r="J35" s="3"/>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A36" s="6"/>
-      <c r="B36" s="6"/>
-      <c r="C36" s="9"/>
-      <c r="D36" s="6"/>
-      <c r="E36" s="9"/>
-      <c r="F36" s="6"/>
-      <c r="G36" s="3"/>
-      <c r="H36" s="3"/>
-      <c r="I36" s="3"/>
-      <c r="J36" s="3"/>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A37" s="2"/>
-      <c r="B37" s="2"/>
-      <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
-      <c r="E37" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="F37" s="5">
-        <f>SUM(F3:F36)</f>
-        <v>87.25</v>
-      </c>
-      <c r="G37" s="5">
-        <f>SUM(G3:G36)</f>
+      <c r="G43">
+        <f>SUMIF(A3:A34, F43,G3:G34)</f>
         <v>4</v>
-      </c>
-      <c r="H37" s="5">
-        <f>SUM(H3:H36)</f>
-        <v>0</v>
-      </c>
-      <c r="I37" s="5">
-        <f>SUM(I3:I36)</f>
-        <v>0</v>
-      </c>
-      <c r="J37" s="5">
-        <f>SUM(J3:J36)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="F38">
-        <v>96</v>
-      </c>
-      <c r="G38">
-        <f>$F$37</f>
-        <v>87.25</v>
-      </c>
-      <c r="H38">
-        <f t="shared" ref="H38:J38" si="0">$F$37</f>
-        <v>87.25</v>
-      </c>
-      <c r="I38">
-        <f t="shared" si="0"/>
-        <v>87.25</v>
-      </c>
-      <c r="J38">
-        <f t="shared" si="0"/>
-        <v>87.25</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="E40" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="F40" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="G40" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="H40" s="7" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="E41" t="s">
-        <v>37</v>
-      </c>
-      <c r="F41">
-        <f>SUMIF(A3:A36, E41,F3:F36)</f>
-        <v>19</v>
-      </c>
-      <c r="G41">
-        <v>24</v>
-      </c>
-      <c r="H41">
-        <f>G41-F41-F45</f>
-        <v>0.75</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="E42" t="s">
-        <v>38</v>
-      </c>
-      <c r="F42">
-        <f>SUMIF(A3:A36, E42,F3:F36)</f>
-        <v>21.25</v>
-      </c>
-      <c r="G42">
-        <v>24</v>
-      </c>
-      <c r="H42">
-        <f>G42-F42-F45</f>
-        <v>-1.5</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="E43" t="s">
-        <v>36</v>
-      </c>
-      <c r="F43">
-        <f>SUMIF(A3:A36, E43,F3:F36)</f>
-        <v>21.75</v>
-      </c>
-      <c r="G43">
-        <v>24</v>
-      </c>
-      <c r="H43">
-        <f>G43-F43-F45</f>
-        <v>-2</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="E44" t="s">
-        <v>39</v>
-      </c>
-      <c r="F44">
-        <f>SUMIF(A3:A36, E44,F3:F36)</f>
-        <v>21</v>
-      </c>
-      <c r="G44">
-        <v>24</v>
-      </c>
-      <c r="H44">
-        <f>G44-F44-F45</f>
-        <v>-1.25</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="E45" t="s">
-        <v>18</v>
-      </c>
-      <c r="F45">
-        <f>SUMIF(A3:A36, E45,F3:F36)</f>
-        <v>4.25</v>
       </c>
     </row>
   </sheetData>
@@ -2525,14 +2563,15 @@
     <sortCondition ref="C3:C36"/>
     <sortCondition ref="E3:E36"/>
   </sortState>
-  <mergeCells count="7">
-    <mergeCell ref="G1:J1"/>
+  <mergeCells count="8">
     <mergeCell ref="F1:F2"/>
     <mergeCell ref="E1:E2"/>
     <mergeCell ref="D1:D2"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="B1:B2"/>
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="H1:K1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Added the Communication Protocols to the Notes
I added the request and response for all the communication protocols
to the sprint Planning Meeting Notes.
</commit_message>
<xml_diff>
--- a/sprints/sprint2/Sprint Backlog & Burnup Chart.xlsx
+++ b/sprints/sprint2/Sprint Backlog & Burnup Chart.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\OneDrive\Documents\College Docs\Software Engineering II\Project\Group5NutritionTracker\sprints\sprint2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\College Docs\Software Engineering II\Project\Group5NutritionTracker\sprints\sprint2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C816719-D512-4BE4-A2F0-38D39455C072}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1753E291-32AF-401D-8137-1C4BBF78B56A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="58">
   <si>
     <t>Related User Story</t>
   </si>
@@ -104,9 +104,6 @@
     <t>Create Account Page Code Behind</t>
   </si>
   <si>
-    <t>Display User Info on Landing After Creation</t>
-  </si>
-  <si>
     <t>Communication Protecol for Create Account</t>
   </si>
   <si>
@@ -122,15 +119,9 @@
     <t>Search Process Server Side</t>
   </si>
   <si>
-    <t>DayOfFood Structure</t>
-  </si>
-  <si>
     <t>Hookup Remove Buttons to User</t>
   </si>
   <si>
-    <t>Credentials Structure</t>
-  </si>
-  <si>
     <t>Communication Protecol for Search</t>
   </si>
   <si>
@@ -140,9 +131,6 @@
     <t>Update DayOfFood Process Server Side</t>
   </si>
   <si>
-    <t>Communication Protecol for Update DayOfFood</t>
-  </si>
-  <si>
     <t>Hookup Add Buttons to Search Page</t>
   </si>
   <si>
@@ -213,6 +201,15 @@
   </si>
   <si>
     <t>Completed By</t>
+  </si>
+  <si>
+    <t>Updated To</t>
+  </si>
+  <si>
+    <t>Communication Protecol for Update FoodLog</t>
+  </si>
+  <si>
+    <t>FoodLog Structure</t>
   </si>
 </sst>
 </file>
@@ -281,7 +278,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -339,7 +336,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -355,28 +352,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -472,6 +463,9 @@
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
+          <c:tx>
+            <c:v>Actual Values</c:v>
+          </c:tx>
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
@@ -486,21 +480,21 @@
           </c:marker>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$G$37:$J$37</c:f>
+              <c:f>Sheet1!$H$35:$K$35</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>4</c:v>
+                  <c:v>4.5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>14.25</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>17.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>17.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -515,6 +509,9 @@
         <c:ser>
           <c:idx val="1"/>
           <c:order val="1"/>
+          <c:tx>
+            <c:v>Goal Line</c:v>
+          </c:tx>
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
@@ -529,21 +526,21 @@
           </c:marker>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$G$38:$J$38</c:f>
+              <c:f>Sheet1!$H$36:$K$36</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>87.25</c:v>
+                  <c:v>84.5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>87.25</c:v>
+                  <c:v>84.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>87.25</c:v>
+                  <c:v>84.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>87.25</c:v>
+                  <c:v>84.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1585,939 +1582,980 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J45"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:K43"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.21875" customWidth="1"/>
-    <col min="3" max="3" width="11.5546875" customWidth="1"/>
-    <col min="4" max="4" width="51.44140625" customWidth="1"/>
+    <col min="1" max="1" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11" customWidth="1"/>
     <col min="5" max="5" width="44" customWidth="1"/>
-    <col min="6" max="6" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.88671875" customWidth="1"/>
+    <col min="6" max="6" width="46.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="C1" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="D1" s="11" t="s">
+      <c r="B1" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="F1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="G1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="10" t="s">
+      <c r="H1" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
-      <c r="J1" s="10"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="12"/>
-      <c r="B2" s="16"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="1" t="s">
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" s="11"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="9">
+      <c r="B3" s="14"/>
+      <c r="C3" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="14">
         <v>1.1000000000000001</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="E3" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="F3" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="F3" s="6">
+      <c r="G3" s="6">
         <v>0.75</v>
       </c>
-      <c r="G3" s="3"/>
       <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
+      <c r="I3" s="3">
+        <v>0.5</v>
+      </c>
       <c r="J3" s="3"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K3" s="3"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="6"/>
-      <c r="C4" s="9">
+      <c r="B4" s="14"/>
+      <c r="C4" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="14">
         <v>1.1000000000000001</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="E4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="F4" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="F4" s="6">
+      <c r="G4" s="6">
         <v>0.25</v>
       </c>
-      <c r="G4" s="3"/>
       <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
+      <c r="I4" s="3">
+        <v>0.25</v>
+      </c>
       <c r="J4" s="3"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K4" s="3"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B5" s="6"/>
-      <c r="C5" s="9">
+        <v>34</v>
+      </c>
+      <c r="B5" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5" s="14">
         <v>1.2</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="E5" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="F5" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="6">
+      <c r="G5" s="6">
         <v>4</v>
       </c>
-      <c r="G5" s="3">
+      <c r="H5" s="3"/>
+      <c r="I5" s="3">
+        <v>6</v>
+      </c>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" s="14"/>
+      <c r="C6" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" s="14">
+        <v>1.2</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F6" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" s="6">
         <v>4</v>
       </c>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="B6" s="6"/>
-      <c r="C6" s="9">
+      <c r="H6" s="3">
+        <v>4</v>
+      </c>
+      <c r="I6" s="3">
+        <v>3</v>
+      </c>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" s="14"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="14">
         <v>1.2</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="E7" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="6">
-        <v>4</v>
-      </c>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
-      <c r="J6" s="3"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B7" s="6"/>
-      <c r="C7" s="9">
-        <v>1.2</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="E7" s="9" t="s">
+      <c r="F7" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="6">
+      <c r="G7" s="6">
         <v>2.5</v>
       </c>
-      <c r="G7" s="3"/>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K7" s="3"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="B8" s="6"/>
-      <c r="C8" s="9">
+        <v>32</v>
+      </c>
+      <c r="B8" s="14"/>
+      <c r="C8" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" s="14">
         <v>1.2</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="E8" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="F8" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="F8" s="6">
+      <c r="G8" s="6">
         <v>2.75</v>
       </c>
-      <c r="G8" s="3"/>
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
       <c r="J8" s="3"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K8" s="3"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="B9" s="6"/>
-      <c r="C9" s="9">
+        <v>32</v>
+      </c>
+      <c r="B9" s="14"/>
+      <c r="C9" s="6"/>
+      <c r="D9" s="14">
         <v>1.3</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="E9" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="F9" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="F9" s="6">
+      <c r="G9" s="6">
         <v>4</v>
       </c>
-      <c r="G9" s="3"/>
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K9" s="3"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="6"/>
-      <c r="C10" s="9">
+      <c r="B10" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" s="14">
         <v>2.1</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="E10" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E10" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="F10" s="6">
+      <c r="F10" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="G10" s="6">
         <v>0.5</v>
       </c>
-      <c r="G10" s="3"/>
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J10" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="K10" s="3"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" s="6"/>
-      <c r="C11" s="9">
-        <v>2.1</v>
-      </c>
-      <c r="D11" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" s="6"/>
+      <c r="D11" s="14">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="E11" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E11" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="F11" s="6">
-        <v>0.25</v>
-      </c>
-      <c r="G11" s="3"/>
+      <c r="F11" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="G11" s="6">
+        <v>4</v>
+      </c>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
       <c r="J11" s="3"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K11" s="3"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B12" s="6"/>
-      <c r="C12" s="9">
+        <v>32</v>
+      </c>
+      <c r="B12" s="14"/>
+      <c r="C12" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D12" s="14">
         <v>2.2000000000000002</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="E12" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E12" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="F12" s="6">
-        <v>2.75</v>
-      </c>
-      <c r="G12" s="3"/>
+      <c r="F12" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="G12" s="6">
+        <v>4</v>
+      </c>
       <c r="H12" s="3"/>
       <c r="I12" s="3"/>
       <c r="J12" s="3"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K12" s="3"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="B13" s="6"/>
-      <c r="C13" s="9">
+        <v>34</v>
+      </c>
+      <c r="B13" s="14"/>
+      <c r="C13" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D13" s="14">
         <v>2.2000000000000002</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="E13" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E13" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="F13" s="6">
-        <v>4</v>
-      </c>
-      <c r="G13" s="3"/>
+      <c r="F13" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="G13" s="6">
+        <v>2.75</v>
+      </c>
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
       <c r="J13" s="3"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K13" s="3"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="B14" s="6"/>
-      <c r="C14" s="9">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="D14" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B14" s="14"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="14">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="E14" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E14" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="F14" s="6">
+      <c r="F14" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="G14" s="6">
         <v>4</v>
       </c>
-      <c r="G14" s="3"/>
       <c r="H14" s="3"/>
       <c r="I14" s="3"/>
       <c r="J14" s="3"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K14" s="3"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B15" s="6"/>
-      <c r="C15" s="9">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E15" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="F15" s="6">
-        <v>2.5</v>
-      </c>
-      <c r="G15" s="3"/>
+        <v>18</v>
+      </c>
+      <c r="B15" s="14"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="14">
+        <v>3.1</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="F15" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="G15" s="6">
+        <v>0.5</v>
+      </c>
       <c r="H15" s="3"/>
       <c r="I15" s="3"/>
       <c r="J15" s="3"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K15" s="3"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B16" s="6"/>
-      <c r="C16" s="9">
-        <v>2.2999999999999998</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E16" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="F16" s="6">
+        <v>32</v>
+      </c>
+      <c r="B16" s="14"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="14">
+        <v>3.2</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="F16" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="G16" s="6">
         <v>4</v>
       </c>
-      <c r="G16" s="3"/>
       <c r="H16" s="3"/>
       <c r="I16" s="3"/>
       <c r="J16" s="3"/>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K16" s="3"/>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="B17" s="6"/>
-      <c r="C17" s="9">
+        <v>35</v>
+      </c>
+      <c r="B17" s="14"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="14">
         <v>3.2</v>
       </c>
-      <c r="D17" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="E17" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="F17" s="6">
+      <c r="E17" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="F17" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="G17" s="6">
         <v>4</v>
       </c>
-      <c r="G17" s="3"/>
       <c r="H17" s="3"/>
       <c r="I17" s="3"/>
       <c r="J17" s="3"/>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K17" s="3"/>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B18" s="6"/>
-      <c r="C18" s="9">
-        <v>3.2</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="E18" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="F18" s="6">
-        <v>4</v>
-      </c>
-      <c r="G18" s="3"/>
+        <v>18</v>
+      </c>
+      <c r="B18" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D18" s="14">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F18" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="G18" s="6">
+        <v>0.5</v>
+      </c>
       <c r="H18" s="3"/>
       <c r="I18" s="3"/>
-      <c r="J18" s="3"/>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J18" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="K18" s="3"/>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="6"/>
-      <c r="C19" s="9">
-        <v>3.1</v>
-      </c>
-      <c r="D19" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="E19" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="F19" s="6">
+      <c r="B19" s="14"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="14">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F19" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="G19" s="6">
         <v>0.5</v>
       </c>
-      <c r="G19" s="3"/>
       <c r="H19" s="3"/>
       <c r="I19" s="3"/>
       <c r="J19" s="3"/>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K19" s="3"/>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="6"/>
-      <c r="C20" s="9">
+      <c r="B20" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D20" s="14">
         <v>4.0999999999999996</v>
       </c>
-      <c r="D20" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E20" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="F20" s="6">
+      <c r="E20" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F20" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="G20" s="6">
         <v>0.5</v>
       </c>
-      <c r="G20" s="3"/>
-      <c r="H20" s="3"/>
+      <c r="H20" s="3">
+        <v>0.5</v>
+      </c>
       <c r="I20" s="3"/>
       <c r="J20" s="3"/>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K20" s="3"/>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B21" s="6"/>
-      <c r="C21" s="9">
-        <v>4.0999999999999996</v>
-      </c>
-      <c r="D21" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B21" s="14"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="14">
+        <v>4.2</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F21" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="E21" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="F21" s="6">
+      <c r="G21" s="6">
         <v>0.5</v>
       </c>
-      <c r="G21" s="3"/>
       <c r="H21" s="3"/>
       <c r="I21" s="3"/>
       <c r="J21" s="3"/>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K21" s="3"/>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B22" s="6"/>
-      <c r="C22" s="9">
-        <v>4.0999999999999996</v>
-      </c>
-      <c r="D22" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E22" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="F22" s="6">
-        <v>0.5</v>
-      </c>
-      <c r="G22" s="3"/>
+        <v>34</v>
+      </c>
+      <c r="B22" s="14"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="14">
+        <v>4.2</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F22" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="G22" s="6">
+        <v>3</v>
+      </c>
       <c r="H22" s="3"/>
       <c r="I22" s="3"/>
       <c r="J22" s="3"/>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K22" s="3"/>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B23" s="6"/>
-      <c r="C23" s="9">
+        <v>32</v>
+      </c>
+      <c r="B23" s="14"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="14">
         <v>4.2</v>
       </c>
-      <c r="D23" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E23" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="F23" s="6">
-        <v>0.5</v>
-      </c>
-      <c r="G23" s="3"/>
+      <c r="E23" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F23" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="G23" s="6">
+        <v>3</v>
+      </c>
       <c r="H23" s="3"/>
       <c r="I23" s="3"/>
       <c r="J23" s="3"/>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K23" s="3"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B24" s="6"/>
-      <c r="C24" s="9">
+        <v>35</v>
+      </c>
+      <c r="B24" s="14"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="14">
         <v>4.2</v>
       </c>
-      <c r="D24" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E24" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="F24" s="6">
-        <v>3</v>
-      </c>
-      <c r="G24" s="3"/>
+      <c r="E24" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F24" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="G24" s="6">
+        <v>4</v>
+      </c>
       <c r="H24" s="3"/>
       <c r="I24" s="3"/>
       <c r="J24" s="3"/>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K24" s="3"/>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="B25" s="6"/>
-      <c r="C25" s="9">
+        <v>33</v>
+      </c>
+      <c r="B25" s="14"/>
+      <c r="C25" s="6"/>
+      <c r="D25" s="14">
         <v>4.2</v>
       </c>
-      <c r="D25" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E25" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="F25" s="6">
-        <v>3</v>
-      </c>
-      <c r="G25" s="3"/>
+      <c r="E25" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F25" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="G25" s="6">
+        <v>4</v>
+      </c>
       <c r="H25" s="3"/>
       <c r="I25" s="3"/>
-      <c r="J25" s="3"/>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J25" s="3">
+        <v>2.5</v>
+      </c>
+      <c r="K25" s="3"/>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B26" s="6"/>
-      <c r="C26" s="9">
-        <v>4.2</v>
-      </c>
-      <c r="D26" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E26" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="F26" s="6">
+        <v>33</v>
+      </c>
+      <c r="B26" s="14"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="14">
+        <v>4.3</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F26" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="G26" s="6">
         <v>4</v>
       </c>
-      <c r="G26" s="3"/>
       <c r="H26" s="3"/>
       <c r="I26" s="3"/>
       <c r="J26" s="3"/>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K26" s="3"/>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="B27" s="6"/>
-      <c r="C27" s="9">
-        <v>4.2</v>
-      </c>
-      <c r="D27" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E27" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="F27" s="6">
+        <v>35</v>
+      </c>
+      <c r="B27" s="14"/>
+      <c r="C27" s="6"/>
+      <c r="D27" s="14">
+        <v>4.3</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F27" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="G27" s="6">
         <v>4</v>
       </c>
-      <c r="G27" s="3"/>
       <c r="H27" s="3"/>
       <c r="I27" s="3"/>
       <c r="J27" s="3"/>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K27" s="3"/>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="B28" s="6"/>
-      <c r="C28" s="9">
-        <v>4.3</v>
-      </c>
-      <c r="D28" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E28" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="F28" s="6">
-        <v>4</v>
-      </c>
-      <c r="G28" s="3"/>
+        <v>18</v>
+      </c>
+      <c r="B28" s="14"/>
+      <c r="C28" s="6"/>
+      <c r="D28" s="14">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="F28" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="G28" s="6">
+        <v>0.5</v>
+      </c>
       <c r="H28" s="3"/>
       <c r="I28" s="3"/>
       <c r="J28" s="3"/>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K28" s="3"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B29" s="6"/>
-      <c r="C29" s="9">
-        <v>4.3</v>
-      </c>
-      <c r="D29" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E29" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="F29" s="6">
-        <v>4</v>
-      </c>
-      <c r="G29" s="3"/>
+        <v>34</v>
+      </c>
+      <c r="B29" s="14"/>
+      <c r="C29" s="6"/>
+      <c r="D29" s="14">
+        <v>5.2</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="F29" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="G29" s="6">
+        <v>5</v>
+      </c>
       <c r="H29" s="3"/>
       <c r="I29" s="3"/>
       <c r="J29" s="3"/>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K29" s="3"/>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B30" s="6"/>
-      <c r="C30" s="9">
+        <v>35</v>
+      </c>
+      <c r="B30" s="14"/>
+      <c r="C30" s="6"/>
+      <c r="D30" s="14">
         <v>5.2</v>
       </c>
-      <c r="D30" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="E30" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="F30" s="6">
-        <v>2</v>
-      </c>
-      <c r="G30" s="3"/>
+      <c r="E30" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="F30" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="G30" s="6">
+        <v>4</v>
+      </c>
       <c r="H30" s="3"/>
       <c r="I30" s="3"/>
       <c r="J30" s="3"/>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K30" s="3"/>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B31" s="6"/>
-      <c r="C31" s="9">
+        <v>32</v>
+      </c>
+      <c r="B31" s="14"/>
+      <c r="C31" s="6"/>
+      <c r="D31" s="14">
         <v>5.2</v>
       </c>
-      <c r="D31" s="6" t="s">
+      <c r="E31" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="F31" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="E31" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="F31" s="6">
-        <v>5</v>
-      </c>
-      <c r="G31" s="3"/>
+      <c r="G31" s="6">
+        <v>4</v>
+      </c>
       <c r="H31" s="3"/>
       <c r="I31" s="3"/>
       <c r="J31" s="3"/>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K31" s="3"/>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="B32" s="6"/>
-      <c r="C32" s="9">
-        <v>5.3</v>
-      </c>
-      <c r="D32" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="E32" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="F32" s="6">
-        <v>3</v>
-      </c>
-      <c r="G32" s="3"/>
+        <v>34</v>
+      </c>
+      <c r="B32" s="14"/>
+      <c r="C32" s="6"/>
+      <c r="D32" s="14">
+        <v>5.2</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="F32" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="G32" s="6">
+        <v>2</v>
+      </c>
       <c r="H32" s="3"/>
       <c r="I32" s="3"/>
       <c r="J32" s="3"/>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K32" s="3"/>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B33" s="6"/>
-      <c r="C33" s="9">
-        <v>5.2</v>
-      </c>
-      <c r="D33" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="E33" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="F33" s="6">
-        <v>4</v>
-      </c>
-      <c r="G33" s="3"/>
+        <v>33</v>
+      </c>
+      <c r="B33" s="14"/>
+      <c r="C33" s="6"/>
+      <c r="D33" s="14">
+        <v>5.3</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="F33" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="G33" s="6">
+        <v>3</v>
+      </c>
       <c r="H33" s="3"/>
       <c r="I33" s="3"/>
       <c r="J33" s="3"/>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A34" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="B34" s="6"/>
-      <c r="C34" s="9">
-        <v>5.2</v>
-      </c>
-      <c r="D34" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="E34" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="F34" s="6">
-        <v>4</v>
-      </c>
-      <c r="G34" s="3"/>
+      <c r="K33" s="3"/>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" s="6"/>
+      <c r="B34" s="14"/>
+      <c r="C34" s="6"/>
+      <c r="D34" s="14"/>
+      <c r="E34" s="6"/>
+      <c r="F34" s="14"/>
+      <c r="G34" s="6"/>
       <c r="H34" s="3"/>
       <c r="I34" s="3"/>
       <c r="J34" s="3"/>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A35" s="6" t="s">
+      <c r="K34" s="3"/>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35" s="2"/>
+      <c r="B35" s="2"/>
+      <c r="C35" s="2"/>
+      <c r="D35" s="2"/>
+      <c r="E35" s="2"/>
+      <c r="F35" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="G35" s="5">
+        <f>SUM(G3:G34)</f>
+        <v>84.5</v>
+      </c>
+      <c r="H35" s="5">
+        <f>SUM(H3:H34)</f>
+        <v>4.5</v>
+      </c>
+      <c r="I35" s="5">
+        <f>SUM(I3:I34, H35)</f>
+        <v>14.25</v>
+      </c>
+      <c r="J35" s="5">
+        <f>SUM(J3:J34, I35)</f>
+        <v>17.5</v>
+      </c>
+      <c r="K35" s="5">
+        <f>SUM(K3:K34, J35)</f>
+        <v>17.5</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="G36">
+        <v>96</v>
+      </c>
+      <c r="H36">
+        <f>$G$35</f>
+        <v>84.5</v>
+      </c>
+      <c r="I36">
+        <f t="shared" ref="I36:K36" si="0">$G$35</f>
+        <v>84.5</v>
+      </c>
+      <c r="J36">
+        <f t="shared" si="0"/>
+        <v>84.5</v>
+      </c>
+      <c r="K36">
+        <f t="shared" si="0"/>
+        <v>84.5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="F38" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G38" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="H38" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="I38" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="J38" s="8"/>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="F39" t="s">
+        <v>33</v>
+      </c>
+      <c r="G39">
+        <f>SUMIF(A3:A34, F39,G3:G34)</f>
+        <v>19</v>
+      </c>
+      <c r="H39">
+        <v>24</v>
+      </c>
+      <c r="I39">
+        <f>H39-G39-G43</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="F40" t="s">
+        <v>34</v>
+      </c>
+      <c r="G40">
+        <f>SUMIF(A3:A34, F40,G3:G34)</f>
+        <v>21.25</v>
+      </c>
+      <c r="H40">
+        <v>24</v>
+      </c>
+      <c r="I40">
+        <f>H40-G40-G43</f>
+        <v>-1.25</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="F41" t="s">
+        <v>32</v>
+      </c>
+      <c r="G41">
+        <f>SUMIF(A3:A34, F41,G3:G34)</f>
+        <v>21.75</v>
+      </c>
+      <c r="H41">
+        <v>24</v>
+      </c>
+      <c r="I41">
+        <f>H41-G41-G43</f>
+        <v>-1.75</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="F42" t="s">
+        <v>35</v>
+      </c>
+      <c r="G42">
+        <f>SUMIF(A3:A34, F42,G3:G34)</f>
+        <v>18.5</v>
+      </c>
+      <c r="H42">
+        <v>24</v>
+      </c>
+      <c r="I42">
+        <f>H42-G42-G43</f>
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="F43" t="s">
         <v>18</v>
       </c>
-      <c r="B35" s="6"/>
-      <c r="C35" s="9">
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="D35" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="E35" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="F35" s="6">
-        <v>0.5</v>
-      </c>
-      <c r="G35" s="3"/>
-      <c r="H35" s="3"/>
-      <c r="I35" s="3"/>
-      <c r="J35" s="3"/>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A36" s="6"/>
-      <c r="B36" s="6"/>
-      <c r="C36" s="9"/>
-      <c r="D36" s="6"/>
-      <c r="E36" s="9"/>
-      <c r="F36" s="6"/>
-      <c r="G36" s="3"/>
-      <c r="H36" s="3"/>
-      <c r="I36" s="3"/>
-      <c r="J36" s="3"/>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A37" s="2"/>
-      <c r="B37" s="2"/>
-      <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
-      <c r="E37" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="F37" s="5">
-        <f>SUM(F3:F36)</f>
-        <v>87.25</v>
-      </c>
-      <c r="G37" s="5">
-        <f>SUM(G3:G36)</f>
+      <c r="G43">
+        <f>SUMIF(A3:A34, F43,G3:G34)</f>
         <v>4</v>
-      </c>
-      <c r="H37" s="5">
-        <f>SUM(H3:H36)</f>
-        <v>0</v>
-      </c>
-      <c r="I37" s="5">
-        <f>SUM(I3:I36)</f>
-        <v>0</v>
-      </c>
-      <c r="J37" s="5">
-        <f>SUM(J3:J36)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="F38">
-        <v>96</v>
-      </c>
-      <c r="G38">
-        <f>$F$37</f>
-        <v>87.25</v>
-      </c>
-      <c r="H38">
-        <f t="shared" ref="H38:J38" si="0">$F$37</f>
-        <v>87.25</v>
-      </c>
-      <c r="I38">
-        <f t="shared" si="0"/>
-        <v>87.25</v>
-      </c>
-      <c r="J38">
-        <f t="shared" si="0"/>
-        <v>87.25</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="E40" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="F40" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="G40" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="H40" s="7" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="E41" t="s">
-        <v>37</v>
-      </c>
-      <c r="F41">
-        <f>SUMIF(A3:A36, E41,F3:F36)</f>
-        <v>19</v>
-      </c>
-      <c r="G41">
-        <v>24</v>
-      </c>
-      <c r="H41">
-        <f>G41-F41-F45</f>
-        <v>0.75</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="E42" t="s">
-        <v>38</v>
-      </c>
-      <c r="F42">
-        <f>SUMIF(A3:A36, E42,F3:F36)</f>
-        <v>21.25</v>
-      </c>
-      <c r="G42">
-        <v>24</v>
-      </c>
-      <c r="H42">
-        <f>G42-F42-F45</f>
-        <v>-1.5</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="E43" t="s">
-        <v>36</v>
-      </c>
-      <c r="F43">
-        <f>SUMIF(A3:A36, E43,F3:F36)</f>
-        <v>21.75</v>
-      </c>
-      <c r="G43">
-        <v>24</v>
-      </c>
-      <c r="H43">
-        <f>G43-F43-F45</f>
-        <v>-2</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="E44" t="s">
-        <v>39</v>
-      </c>
-      <c r="F44">
-        <f>SUMIF(A3:A36, E44,F3:F36)</f>
-        <v>21</v>
-      </c>
-      <c r="G44">
-        <v>24</v>
-      </c>
-      <c r="H44">
-        <f>G44-F44-F45</f>
-        <v>-1.25</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="E45" t="s">
-        <v>18</v>
-      </c>
-      <c r="F45">
-        <f>SUMIF(A3:A36, E45,F3:F36)</f>
-        <v>4.25</v>
       </c>
     </row>
   </sheetData>
@@ -2525,14 +2563,15 @@
     <sortCondition ref="C3:C36"/>
     <sortCondition ref="E3:E36"/>
   </sortState>
-  <mergeCells count="7">
-    <mergeCell ref="G1:J1"/>
+  <mergeCells count="8">
     <mergeCell ref="F1:F2"/>
     <mergeCell ref="E1:E2"/>
     <mergeCell ref="D1:D2"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="B1:B2"/>
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="H1:K1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Added Sprint Retrospective Updated Backlog
I added the sprint retrospective from our meeting.
I updated the Sprint Backlog to the most recent info.
</commit_message>
<xml_diff>
--- a/sprints/sprint2/Sprint Backlog & Burnup Chart.xlsx
+++ b/sprints/sprint2/Sprint Backlog & Burnup Chart.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\College Docs\Software Engineering II\Project\Group5NutritionTracker\sprints\sprint2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1753E291-32AF-401D-8137-1C4BBF78B56A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB5420D6-92E7-4928-B162-03769DE16618}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="58">
   <si>
     <t>Related User Story</t>
   </si>
@@ -352,13 +352,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -367,7 +362,12 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -491,10 +491,10 @@
                   <c:v>14.25</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>17.5</c:v>
+                  <c:v>21.75</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>17.5</c:v>
+                  <c:v>23.75</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1596,16 +1596,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="11" t="s">
         <v>40</v>
       </c>
       <c r="E1" s="10" t="s">
@@ -1617,18 +1617,18 @@
       <c r="G1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="H1" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
-      <c r="K1" s="9"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="14"/>
+      <c r="K1" s="14"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="11"/>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
+      <c r="A2" s="13"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
       <c r="E2" s="10"/>
       <c r="F2" s="10"/>
       <c r="G2" s="10"/>
@@ -1649,17 +1649,17 @@
       <c r="A3" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="14"/>
+      <c r="B3" s="9"/>
       <c r="C3" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="14">
+      <c r="D3" s="9">
         <v>1.1000000000000001</v>
       </c>
       <c r="E3" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="14" t="s">
+      <c r="F3" s="9" t="s">
         <v>16</v>
       </c>
       <c r="G3" s="6">
@@ -1676,17 +1676,17 @@
       <c r="A4" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="14"/>
+      <c r="B4" s="9"/>
       <c r="C4" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="14">
+      <c r="D4" s="9">
         <v>1.1000000000000001</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="9" t="s">
         <v>15</v>
       </c>
       <c r="G4" s="6">
@@ -1703,19 +1703,19 @@
       <c r="A5" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="9" t="s">
         <v>33</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="14">
+      <c r="D5" s="9">
         <v>1.2</v>
       </c>
       <c r="E5" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="14" t="s">
+      <c r="F5" s="9" t="s">
         <v>11</v>
       </c>
       <c r="G5" s="6">
@@ -1732,17 +1732,17 @@
       <c r="A6" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B6" s="14"/>
+      <c r="B6" s="9"/>
       <c r="C6" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="D6" s="14">
+      <c r="D6" s="9">
         <v>1.2</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="F6" s="9" t="s">
         <v>12</v>
       </c>
       <c r="G6" s="6">
@@ -1761,15 +1761,17 @@
       <c r="A7" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B7" s="14"/>
-      <c r="C7" s="6"/>
-      <c r="D7" s="14">
+      <c r="B7" s="9"/>
+      <c r="C7" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" s="9">
         <v>1.2</v>
       </c>
       <c r="E7" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="14" t="s">
+      <c r="F7" s="9" t="s">
         <v>14</v>
       </c>
       <c r="G7" s="6">
@@ -1784,17 +1786,17 @@
       <c r="A8" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="14"/>
+      <c r="B8" s="9"/>
       <c r="C8" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D8" s="14">
+      <c r="D8" s="9">
         <v>1.2</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F8" s="14" t="s">
+      <c r="F8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="G8" s="6">
@@ -1809,15 +1811,17 @@
       <c r="A9" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B9" s="14"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="14">
+      <c r="B9" s="9"/>
+      <c r="C9" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" s="9">
         <v>1.3</v>
       </c>
       <c r="E9" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F9" s="14" t="s">
+      <c r="F9" s="9" t="s">
         <v>13</v>
       </c>
       <c r="G9" s="6">
@@ -1832,19 +1836,19 @@
       <c r="A10" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="9" t="s">
         <v>33</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="D10" s="14">
+      <c r="D10" s="9">
         <v>2.1</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F10" s="14" t="s">
+      <c r="F10" s="9" t="s">
         <v>22</v>
       </c>
       <c r="G10" s="6">
@@ -1861,17 +1865,17 @@
       <c r="A11" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B11" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="C11" s="6"/>
-      <c r="D11" s="14">
+      <c r="B11" s="9"/>
+      <c r="C11" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D11" s="9">
         <v>2.2000000000000002</v>
       </c>
       <c r="E11" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F11" s="14" t="s">
+      <c r="F11" s="9" t="s">
         <v>51</v>
       </c>
       <c r="G11" s="6">
@@ -1879,24 +1883,26 @@
       </c>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
-      <c r="J11" s="3"/>
+      <c r="J11" s="3">
+        <v>3.5</v>
+      </c>
       <c r="K11" s="3"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B12" s="14"/>
+      <c r="B12" s="9"/>
       <c r="C12" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D12" s="14">
+      <c r="D12" s="9">
         <v>2.2000000000000002</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F12" s="14" t="s">
+      <c r="F12" s="9" t="s">
         <v>52</v>
       </c>
       <c r="G12" s="6">
@@ -1911,17 +1917,17 @@
       <c r="A13" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="14"/>
+      <c r="B13" s="9"/>
       <c r="C13" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D13" s="14">
+      <c r="D13" s="9">
         <v>2.2000000000000002</v>
       </c>
       <c r="E13" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="14" t="s">
+      <c r="F13" s="9" t="s">
         <v>20</v>
       </c>
       <c r="G13" s="6">
@@ -1936,15 +1942,19 @@
       <c r="A14" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B14" s="14"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="14">
+      <c r="B14" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D14" s="9">
         <v>2.2999999999999998</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F14" s="14" t="s">
+      <c r="F14" s="9" t="s">
         <v>21</v>
       </c>
       <c r="G14" s="6">
@@ -1959,15 +1969,19 @@
       <c r="A15" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="14"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="14">
+      <c r="B15" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D15" s="9">
         <v>3.1</v>
       </c>
       <c r="E15" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="F15" s="14" t="s">
+      <c r="F15" s="9" t="s">
         <v>50</v>
       </c>
       <c r="G15" s="6">
@@ -1975,22 +1989,26 @@
       </c>
       <c r="H15" s="3"/>
       <c r="I15" s="3"/>
-      <c r="J15" s="3"/>
+      <c r="J15" s="3">
+        <v>0.25</v>
+      </c>
       <c r="K15" s="3"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="14"/>
-      <c r="C16" s="6"/>
-      <c r="D16" s="14">
+      <c r="B16" s="9"/>
+      <c r="C16" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D16" s="9">
         <v>3.2</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="F16" s="14" t="s">
+      <c r="F16" s="9" t="s">
         <v>48</v>
       </c>
       <c r="G16" s="6">
@@ -2005,15 +2023,17 @@
       <c r="A17" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B17" s="14"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="14">
+      <c r="B17" s="9"/>
+      <c r="C17" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D17" s="9">
         <v>3.2</v>
       </c>
       <c r="E17" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="F17" s="14" t="s">
+      <c r="F17" s="9" t="s">
         <v>49</v>
       </c>
       <c r="G17" s="6">
@@ -2022,25 +2042,27 @@
       <c r="H17" s="3"/>
       <c r="I17" s="3"/>
       <c r="J17" s="3"/>
-      <c r="K17" s="3"/>
+      <c r="K17" s="3">
+        <v>2</v>
+      </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B18" s="14" t="s">
+      <c r="B18" s="9" t="s">
         <v>33</v>
       </c>
       <c r="C18" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="D18" s="14">
+      <c r="D18" s="9">
         <v>4.0999999999999996</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="F18" s="14" t="s">
+      <c r="F18" s="9" t="s">
         <v>28</v>
       </c>
       <c r="G18" s="6">
@@ -2057,15 +2079,19 @@
       <c r="A19" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="14"/>
-      <c r="C19" s="6"/>
-      <c r="D19" s="14">
+      <c r="B19" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D19" s="9">
         <v>4.0999999999999996</v>
       </c>
       <c r="E19" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="F19" s="14" t="s">
+      <c r="F19" s="9" t="s">
         <v>56</v>
       </c>
       <c r="G19" s="6">
@@ -2073,26 +2099,28 @@
       </c>
       <c r="H19" s="3"/>
       <c r="I19" s="3"/>
-      <c r="J19" s="3"/>
+      <c r="J19" s="3">
+        <v>0.25</v>
+      </c>
       <c r="K19" s="3"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="14" t="s">
+      <c r="B20" s="9" t="s">
         <v>33</v>
       </c>
       <c r="C20" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="D20" s="14">
+      <c r="D20" s="9">
         <v>4.0999999999999996</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="F20" s="14" t="s">
+      <c r="F20" s="9" t="s">
         <v>57</v>
       </c>
       <c r="G20" s="6">
@@ -2109,15 +2137,19 @@
       <c r="A21" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B21" s="14"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="14">
+      <c r="B21" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D21" s="9">
         <v>4.2</v>
       </c>
       <c r="E21" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="F21" s="14" t="s">
+      <c r="F21" s="9" t="s">
         <v>24</v>
       </c>
       <c r="G21" s="6">
@@ -2132,15 +2164,15 @@
       <c r="A22" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B22" s="14"/>
+      <c r="B22" s="9"/>
       <c r="C22" s="6"/>
-      <c r="D22" s="14">
+      <c r="D22" s="9">
         <v>4.2</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="F22" s="14" t="s">
+      <c r="F22" s="9" t="s">
         <v>31</v>
       </c>
       <c r="G22" s="6">
@@ -2155,15 +2187,15 @@
       <c r="A23" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B23" s="14"/>
+      <c r="B23" s="9"/>
       <c r="C23" s="6"/>
-      <c r="D23" s="14">
+      <c r="D23" s="9">
         <v>4.2</v>
       </c>
       <c r="E23" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="F23" s="14" t="s">
+      <c r="F23" s="9" t="s">
         <v>27</v>
       </c>
       <c r="G23" s="6">
@@ -2178,15 +2210,15 @@
       <c r="A24" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B24" s="14"/>
+      <c r="B24" s="9"/>
       <c r="C24" s="6"/>
-      <c r="D24" s="14">
+      <c r="D24" s="9">
         <v>4.2</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="F24" s="14" t="s">
+      <c r="F24" s="9" t="s">
         <v>25</v>
       </c>
       <c r="G24" s="6">
@@ -2201,15 +2233,17 @@
       <c r="A25" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B25" s="14"/>
-      <c r="C25" s="6"/>
-      <c r="D25" s="14">
+      <c r="B25" s="9"/>
+      <c r="C25" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D25" s="9">
         <v>4.2</v>
       </c>
       <c r="E25" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="F25" s="14" t="s">
+      <c r="F25" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G25" s="6">
@@ -2226,15 +2260,17 @@
       <c r="A26" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B26" s="14"/>
+      <c r="B26" s="9" t="s">
+        <v>34</v>
+      </c>
       <c r="C26" s="6"/>
-      <c r="D26" s="14">
+      <c r="D26" s="9">
         <v>4.3</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="F26" s="14" t="s">
+      <c r="F26" s="9" t="s">
         <v>29</v>
       </c>
       <c r="G26" s="6">
@@ -2249,15 +2285,15 @@
       <c r="A27" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B27" s="14"/>
+      <c r="B27" s="9"/>
       <c r="C27" s="6"/>
-      <c r="D27" s="14">
+      <c r="D27" s="9">
         <v>4.3</v>
       </c>
       <c r="E27" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="F27" s="14" t="s">
+      <c r="F27" s="9" t="s">
         <v>30</v>
       </c>
       <c r="G27" s="6">
@@ -2272,15 +2308,19 @@
       <c r="A28" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B28" s="14"/>
-      <c r="C28" s="6"/>
-      <c r="D28" s="14">
+      <c r="B28" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D28" s="9">
         <v>5.0999999999999996</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="F28" s="14" t="s">
+      <c r="F28" s="9" t="s">
         <v>46</v>
       </c>
       <c r="G28" s="6">
@@ -2288,22 +2328,24 @@
       </c>
       <c r="H28" s="3"/>
       <c r="I28" s="3"/>
-      <c r="J28" s="3"/>
+      <c r="J28" s="3">
+        <v>0.25</v>
+      </c>
       <c r="K28" s="3"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B29" s="14"/>
+      <c r="B29" s="9"/>
       <c r="C29" s="6"/>
-      <c r="D29" s="14">
+      <c r="D29" s="9">
         <v>5.2</v>
       </c>
       <c r="E29" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="F29" s="14" t="s">
+      <c r="F29" s="9" t="s">
         <v>53</v>
       </c>
       <c r="G29" s="6">
@@ -2318,15 +2360,15 @@
       <c r="A30" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B30" s="14"/>
+      <c r="B30" s="9"/>
       <c r="C30" s="6"/>
-      <c r="D30" s="14">
+      <c r="D30" s="9">
         <v>5.2</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="F30" s="14" t="s">
+      <c r="F30" s="9" t="s">
         <v>44</v>
       </c>
       <c r="G30" s="6">
@@ -2341,15 +2383,17 @@
       <c r="A31" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B31" s="14"/>
+      <c r="B31" s="9" t="s">
+        <v>34</v>
+      </c>
       <c r="C31" s="6"/>
-      <c r="D31" s="14">
+      <c r="D31" s="9">
         <v>5.2</v>
       </c>
       <c r="E31" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="F31" s="14" t="s">
+      <c r="F31" s="9" t="s">
         <v>45</v>
       </c>
       <c r="G31" s="6">
@@ -2364,15 +2408,15 @@
       <c r="A32" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B32" s="14"/>
+      <c r="B32" s="9"/>
       <c r="C32" s="6"/>
-      <c r="D32" s="14">
+      <c r="D32" s="9">
         <v>5.2</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="F32" s="14" t="s">
+      <c r="F32" s="9" t="s">
         <v>42</v>
       </c>
       <c r="G32" s="6">
@@ -2387,15 +2431,17 @@
       <c r="A33" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B33" s="14"/>
+      <c r="B33" s="9" t="s">
+        <v>35</v>
+      </c>
       <c r="C33" s="6"/>
-      <c r="D33" s="14">
+      <c r="D33" s="9">
         <v>5.3</v>
       </c>
       <c r="E33" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="F33" s="14" t="s">
+      <c r="F33" s="9" t="s">
         <v>43</v>
       </c>
       <c r="G33" s="6">
@@ -2408,11 +2454,11 @@
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="6"/>
-      <c r="B34" s="14"/>
+      <c r="B34" s="9"/>
       <c r="C34" s="6"/>
-      <c r="D34" s="14"/>
+      <c r="D34" s="9"/>
       <c r="E34" s="6"/>
-      <c r="F34" s="14"/>
+      <c r="F34" s="9"/>
       <c r="G34" s="6"/>
       <c r="H34" s="3"/>
       <c r="I34" s="3"/>
@@ -2442,11 +2488,11 @@
       </c>
       <c r="J35" s="5">
         <f>SUM(J3:J34, I35)</f>
-        <v>17.5</v>
+        <v>21.75</v>
       </c>
       <c r="K35" s="5">
         <f>SUM(K3:K34, J35)</f>
-        <v>17.5</v>
+        <v>23.75</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
@@ -2564,14 +2610,14 @@
     <sortCondition ref="E3:E36"/>
   </sortState>
   <mergeCells count="8">
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="H1:K1"/>
     <mergeCell ref="F1:F2"/>
     <mergeCell ref="E1:E2"/>
     <mergeCell ref="D1:D2"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="B1:B2"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="H1:K1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>